<commit_message>
audit batch 2: CI (F-48), migrate-on-deploy (F-49), build id in footer (F-50), mobile nav (F-32), fix onboarding tour (F-33), pipeline maxDuration (F-04)
</commit_message>
<xml_diff>
--- a/docs/BSA_Application_Audit.xlsx
+++ b/docs/BSA_Application_Audit.xlsx
@@ -258,25 +258,25 @@
     <t xml:space="preserve">M</t>
   </si>
   <si>
+    <t xml:space="preserve">F-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two browser tabs (or a double click) can process the same pending sites at the same time.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The orchestrator picks pending sites with a plain read; nothing claims them before processing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claim each site with a conditional updateMany (e.g. set processing_started_at where analyzed_at is null and not recently claimed) and skip sites whose claim fails.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each site is analysed exactly once per run; no duplicated work or racing writes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/modules/orchestrator.ts:117-128</t>
+  </si>
+  <si>
     <t xml:space="preserve">Open</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Two browser tabs (or a double click) can process the same pending sites at the same time.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The orchestrator picks pending sites with a plain read; nothing claims them before processing.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claim each site with a conditional updateMany (e.g. set processing_started_at where analyzed_at is null and not recently claimed) and skip sites whose claim fails.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Each site is analysed exactly once per run; no duplicated work or racing writes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/modules/orchestrator.ts:117-128</t>
   </si>
   <si>
     <t xml:space="preserve">F-06</t>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A6,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="F10" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A10,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="F12" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A12,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="F13" s="9" t="n">
         <f aca="false">SUM(F6:F12)</f>
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2444,12 +2444,12 @@
         <v>57</v>
       </c>
       <c r="M8" s="14" t="s">
-        <v>77</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>9</v>
@@ -2462,19 +2462,19 @@
         <v>P2</v>
       </c>
       <c r="E9" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="F9" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="G9" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="G9" s="15" t="s">
+      <c r="H9" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="H9" s="15" t="s">
+      <c r="I9" s="15" t="s">
         <v>82</v>
-      </c>
-      <c r="I9" s="15" t="s">
-        <v>83</v>
       </c>
       <c r="J9" s="14" t="s">
         <v>76</v>
@@ -2486,7 +2486,7 @@
         <v>57</v>
       </c>
       <c r="M9" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2528,7 +2528,7 @@
         <v>57</v>
       </c>
       <c r="M10" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2612,7 +2612,7 @@
         <v>57</v>
       </c>
       <c r="M12" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2654,7 +2654,7 @@
         <v>57</v>
       </c>
       <c r="M13" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2696,7 +2696,7 @@
         <v>57</v>
       </c>
       <c r="M14" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2738,7 +2738,7 @@
         <v>57</v>
       </c>
       <c r="M15" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2780,7 +2780,7 @@
         <v>57</v>
       </c>
       <c r="M16" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2822,7 +2822,7 @@
         <v>57</v>
       </c>
       <c r="M17" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2864,7 +2864,7 @@
         <v>138</v>
       </c>
       <c r="M18" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2906,7 +2906,7 @@
         <v>145</v>
       </c>
       <c r="M19" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2948,7 +2948,7 @@
         <v>153</v>
       </c>
       <c r="M20" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2990,7 +2990,7 @@
         <v>160</v>
       </c>
       <c r="M21" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3032,7 +3032,7 @@
         <v>167</v>
       </c>
       <c r="M22" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3074,7 +3074,7 @@
         <v>174</v>
       </c>
       <c r="M23" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3116,7 +3116,7 @@
         <v>181</v>
       </c>
       <c r="M24" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3158,7 +3158,7 @@
         <v>57</v>
       </c>
       <c r="M25" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3200,7 +3200,7 @@
         <v>194</v>
       </c>
       <c r="M26" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3242,7 +3242,7 @@
         <v>57</v>
       </c>
       <c r="M27" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3284,7 +3284,7 @@
         <v>57</v>
       </c>
       <c r="M28" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3326,7 +3326,7 @@
         <v>57</v>
       </c>
       <c r="M29" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3368,7 +3368,7 @@
         <v>219</v>
       </c>
       <c r="M30" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3410,7 +3410,7 @@
         <v>57</v>
       </c>
       <c r="M31" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3452,7 +3452,7 @@
         <v>57</v>
       </c>
       <c r="M32" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3494,7 +3494,7 @@
         <v>57</v>
       </c>
       <c r="M33" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3536,7 +3536,7 @@
         <v>244</v>
       </c>
       <c r="M34" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3578,7 +3578,7 @@
         <v>251</v>
       </c>
       <c r="M35" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3620,7 +3620,7 @@
         <v>258</v>
       </c>
       <c r="M36" s="14" t="s">
-        <v>77</v>
+        <v>8</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3662,7 +3662,7 @@
         <v>57</v>
       </c>
       <c r="M37" s="14" t="s">
-        <v>77</v>
+        <v>8</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3704,7 +3704,7 @@
         <v>57</v>
       </c>
       <c r="M38" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3746,7 +3746,7 @@
         <v>57</v>
       </c>
       <c r="M39" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3788,7 +3788,7 @@
         <v>57</v>
       </c>
       <c r="M40" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3830,7 +3830,7 @@
         <v>57</v>
       </c>
       <c r="M41" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3872,7 +3872,7 @@
         <v>57</v>
       </c>
       <c r="M42" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3914,7 +3914,7 @@
         <v>57</v>
       </c>
       <c r="M43" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3956,7 +3956,7 @@
         <v>307</v>
       </c>
       <c r="M44" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3998,7 +3998,7 @@
         <v>57</v>
       </c>
       <c r="M45" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4040,7 +4040,7 @@
         <v>57</v>
       </c>
       <c r="M46" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4082,7 +4082,7 @@
         <v>327</v>
       </c>
       <c r="M47" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4124,7 +4124,7 @@
         <v>57</v>
       </c>
       <c r="M48" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4166,7 +4166,7 @@
         <v>57</v>
       </c>
       <c r="M49" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4208,7 +4208,7 @@
         <v>346</v>
       </c>
       <c r="M50" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4250,7 +4250,7 @@
         <v>353</v>
       </c>
       <c r="M51" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4292,7 +4292,7 @@
         <v>360</v>
       </c>
       <c r="M52" s="14" t="s">
-        <v>77</v>
+        <v>8</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4334,7 +4334,7 @@
         <v>367</v>
       </c>
       <c r="M53" s="14" t="s">
-        <v>77</v>
+        <v>8</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4376,7 +4376,7 @@
         <v>374</v>
       </c>
       <c r="M54" s="14" t="s">
-        <v>77</v>
+        <v>8</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4418,7 +4418,7 @@
         <v>381</v>
       </c>
       <c r="M55" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4460,7 +4460,7 @@
         <v>57</v>
       </c>
       <c r="M56" s="14" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
audit batch 3: remove orphaned pages/components (F-34); partial AI-leftover cleanup (F-42); mark F-35/F-38 done (design pass)
</commit_message>
<xml_diff>
--- a/docs/BSA_Application_Audit.xlsx
+++ b/docs/BSA_Application_Audit.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="419">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="420">
   <si>
     <t xml:space="preserve">BSA v3 — Application Audit</t>
   </si>
@@ -988,6 +988,9 @@
   </si>
   <si>
     <t xml:space="preserve">lib/ai/*; lib/modules/orchestrator.ts:8,113; app/(app)/site/page.tsx:66; prisma/schema.prisma:592-620; .env.example</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In progress</t>
   </si>
   <si>
     <t xml:space="preserve">F-43</t>
@@ -2021,7 +2024,7 @@
       </c>
       <c r="F10" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A10,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2096,7 +2099,7 @@
       </c>
       <c r="F13" s="9" t="n">
         <f aca="false">SUM(F6:F12)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3704,7 +3707,7 @@
         <v>57</v>
       </c>
       <c r="M38" s="14" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3746,7 +3749,7 @@
         <v>57</v>
       </c>
       <c r="M39" s="14" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3872,7 +3875,7 @@
         <v>57</v>
       </c>
       <c r="M42" s="14" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4040,12 +4043,12 @@
         <v>57</v>
       </c>
       <c r="M46" s="14" t="s">
-        <v>83</v>
+        <v>321</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="14" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B47" s="15" t="s">
         <v>14</v>
@@ -4058,19 +4061,19 @@
         <v>P2</v>
       </c>
       <c r="E47" s="15" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F47" s="15" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="G47" s="15" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="H47" s="15" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="I47" s="15" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="J47" s="14" t="s">
         <v>152</v>
@@ -4079,7 +4082,7 @@
         <v>56</v>
       </c>
       <c r="L47" s="15" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="M47" s="14" t="s">
         <v>83</v>
@@ -4087,7 +4090,7 @@
     </row>
     <row r="48" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="14" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B48" s="15" t="s">
         <v>14</v>
@@ -4100,19 +4103,19 @@
         <v>P3</v>
       </c>
       <c r="E48" s="15" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F48" s="15" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="G48" s="15" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="H48" s="15" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="I48" s="15" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="J48" s="14" t="s">
         <v>76</v>
@@ -4129,7 +4132,7 @@
     </row>
     <row r="49" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="14" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B49" s="15" t="s">
         <v>14</v>
@@ -4142,19 +4145,19 @@
         <v>P3</v>
       </c>
       <c r="E49" s="15" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F49" s="15" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="G49" s="15" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="H49" s="15" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="I49" s="15" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="J49" s="14" t="s">
         <v>55</v>
@@ -4171,7 +4174,7 @@
     </row>
     <row r="50" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="14" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B50" s="15" t="s">
         <v>14</v>
@@ -4184,19 +4187,19 @@
         <v>P3</v>
       </c>
       <c r="E50" s="15" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F50" s="15" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G50" s="15" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="H50" s="15" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="I50" s="15" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J50" s="14" t="s">
         <v>55</v>
@@ -4205,7 +4208,7 @@
         <v>56</v>
       </c>
       <c r="L50" s="15" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="M50" s="14" t="s">
         <v>83</v>
@@ -4213,7 +4216,7 @@
     </row>
     <row r="51" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="14" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B51" s="15" t="s">
         <v>14</v>
@@ -4226,19 +4229,19 @@
         <v>P2</v>
       </c>
       <c r="E51" s="15" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F51" s="15" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G51" s="15" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="H51" s="15" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="I51" s="15" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="J51" s="14" t="s">
         <v>76</v>
@@ -4247,7 +4250,7 @@
         <v>56</v>
       </c>
       <c r="L51" s="15" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="M51" s="14" t="s">
         <v>83</v>
@@ -4255,7 +4258,7 @@
     </row>
     <row r="52" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="14" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B52" s="15" t="s">
         <v>15</v>
@@ -4268,19 +4271,19 @@
         <v>P1</v>
       </c>
       <c r="E52" s="15" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F52" s="15" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G52" s="15" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="H52" s="15" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="I52" s="15" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="J52" s="14" t="s">
         <v>55</v>
@@ -4289,7 +4292,7 @@
         <v>56</v>
       </c>
       <c r="L52" s="15" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="M52" s="14" t="s">
         <v>8</v>
@@ -4297,7 +4300,7 @@
     </row>
     <row r="53" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="14" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B53" s="15" t="s">
         <v>15</v>
@@ -4310,19 +4313,19 @@
         <v>P1</v>
       </c>
       <c r="E53" s="15" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F53" s="15" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G53" s="15" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="H53" s="15" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="I53" s="15" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="J53" s="14" t="s">
         <v>55</v>
@@ -4331,7 +4334,7 @@
         <v>56</v>
       </c>
       <c r="L53" s="15" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="M53" s="14" t="s">
         <v>8</v>
@@ -4339,7 +4342,7 @@
     </row>
     <row r="54" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="14" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B54" s="15" t="s">
         <v>15</v>
@@ -4352,19 +4355,19 @@
         <v>P1</v>
       </c>
       <c r="E54" s="15" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F54" s="15" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="G54" s="15" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="H54" s="15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="I54" s="15" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="J54" s="14" t="s">
         <v>76</v>
@@ -4373,7 +4376,7 @@
         <v>56</v>
       </c>
       <c r="L54" s="15" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="M54" s="14" t="s">
         <v>8</v>
@@ -4381,7 +4384,7 @@
     </row>
     <row r="55" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="14" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B55" s="15" t="s">
         <v>15</v>
@@ -4394,19 +4397,19 @@
         <v>P2</v>
       </c>
       <c r="E55" s="15" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F55" s="15" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="G55" s="15" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="H55" s="15" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="I55" s="15" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="J55" s="14" t="s">
         <v>55</v>
@@ -4415,7 +4418,7 @@
         <v>56</v>
       </c>
       <c r="L55" s="15" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="M55" s="14" t="s">
         <v>83</v>
@@ -4423,7 +4426,7 @@
     </row>
     <row r="56" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="14" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B56" s="15" t="s">
         <v>15</v>
@@ -4436,19 +4439,19 @@
         <v>P2</v>
       </c>
       <c r="E56" s="15" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="F56" s="15" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="G56" s="15" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="H56" s="15" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="I56" s="15" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="J56" s="14" t="s">
         <v>55</v>
@@ -4517,7 +4520,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4528,122 +4531,122 @@
         <v>3</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
audit batch 4: per-region rent calibration (F-08), region-aware corridor fallback (F-09), no confident scores from missing data (F-10)
</commit_message>
<xml_diff>
--- a/docs/BSA_Application_Audit.xlsx
+++ b/docs/BSA_Application_Audit.xlsx
@@ -1949,7 +1949,7 @@
       </c>
       <c r="F7" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A7,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="F13" s="9" t="n">
         <f aca="false">SUM(F6:F12)</f>
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2615,7 +2615,7 @@
         <v>57</v>
       </c>
       <c r="M12" s="14" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2657,7 +2657,7 @@
         <v>57</v>
       </c>
       <c r="M13" s="14" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2699,7 +2699,7 @@
         <v>57</v>
       </c>
       <c r="M14" s="14" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
audit batch 5: module_result run index + drop duplicate GiST + migration_lock (F-21); demographic_cell region column (F-12 partial)
</commit_message>
<xml_diff>
--- a/docs/BSA_Application_Audit.xlsx
+++ b/docs/BSA_Application_Audit.xlsx
@@ -405,6 +405,9 @@
     <t xml:space="preserve">prisma/schema.prisma:398-457; lib/ingest/loaders.ts:185</t>
   </si>
   <si>
+    <t xml:space="preserve">In progress</t>
+  </si>
+  <si>
     <t xml:space="preserve">F-13</t>
   </si>
   <si>
@@ -988,9 +991,6 @@
   </si>
   <si>
     <t xml:space="preserve">lib/ai/*; lib/modules/orchestrator.ts:8,113; app/(app)/site/page.tsx:66; prisma/schema.prisma:592-620; .env.example</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In progress</t>
   </si>
   <si>
     <t xml:space="preserve">F-43</t>
@@ -1974,7 +1974,7 @@
       </c>
       <c r="F8" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A8,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="F13" s="9" t="n">
         <f aca="false">SUM(F6:F12)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2783,12 +2783,12 @@
         <v>57</v>
       </c>
       <c r="M16" s="14" t="s">
-        <v>83</v>
+        <v>126</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B17" s="15" t="s">
         <v>10</v>
@@ -2801,19 +2801,19 @@
         <v>P2</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G17" s="15" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H17" s="15" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J17" s="14" t="s">
         <v>55</v>
@@ -2830,7 +2830,7 @@
     </row>
     <row r="18" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>10</v>
@@ -2843,19 +2843,19 @@
         <v>P2</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F18" s="15" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G18" s="15" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I18" s="15" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J18" s="14" t="s">
         <v>76</v>
@@ -2864,7 +2864,7 @@
         <v>56</v>
       </c>
       <c r="L18" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M18" s="14" t="s">
         <v>83</v>
@@ -2872,7 +2872,7 @@
     </row>
     <row r="19" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B19" s="15" t="s">
         <v>10</v>
@@ -2885,19 +2885,19 @@
         <v>P2</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G19" s="15" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H19" s="15" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I19" s="15" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J19" s="14" t="s">
         <v>76</v>
@@ -2906,7 +2906,7 @@
         <v>56</v>
       </c>
       <c r="L19" s="15" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="M19" s="14" t="s">
         <v>83</v>
@@ -2914,7 +2914,7 @@
     </row>
     <row r="20" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B20" s="15" t="s">
         <v>10</v>
@@ -2927,28 +2927,28 @@
         <v>P3</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H20" s="15" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I20" s="15" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J20" s="14" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K20" s="15" t="s">
         <v>56</v>
       </c>
       <c r="L20" s="15" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="M20" s="14" t="s">
         <v>83</v>
@@ -2956,7 +2956,7 @@
     </row>
     <row r="21" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B21" s="15" t="s">
         <v>10</v>
@@ -2969,19 +2969,19 @@
         <v>P3</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G21" s="15" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H21" s="15" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I21" s="15" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J21" s="14" t="s">
         <v>55</v>
@@ -2990,7 +2990,7 @@
         <v>46</v>
       </c>
       <c r="L21" s="15" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="M21" s="14" t="s">
         <v>83</v>
@@ -2998,7 +2998,7 @@
     </row>
     <row r="22" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>10</v>
@@ -3011,19 +3011,19 @@
         <v>P3</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G22" s="15" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H22" s="15" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I22" s="15" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J22" s="14" t="s">
         <v>76</v>
@@ -3032,7 +3032,7 @@
         <v>56</v>
       </c>
       <c r="L22" s="15" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M22" s="14" t="s">
         <v>83</v>
@@ -3040,7 +3040,7 @@
     </row>
     <row r="23" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>10</v>
@@ -3053,28 +3053,28 @@
         <v>P1</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G23" s="15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H23" s="15" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I23" s="15" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J23" s="14" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K23" s="15" t="s">
         <v>46</v>
       </c>
       <c r="L23" s="15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="M23" s="14" t="s">
         <v>83</v>
@@ -3082,7 +3082,7 @@
     </row>
     <row r="24" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>11</v>
@@ -3095,19 +3095,19 @@
         <v>P1</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H24" s="15" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I24" s="15" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J24" s="14" t="s">
         <v>76</v>
@@ -3116,7 +3116,7 @@
         <v>56</v>
       </c>
       <c r="L24" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="M24" s="14" t="s">
         <v>83</v>
@@ -3124,7 +3124,7 @@
     </row>
     <row r="25" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B25" s="15" t="s">
         <v>11</v>
@@ -3137,19 +3137,19 @@
         <v>P2</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G25" s="15" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H25" s="15" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I25" s="15" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J25" s="14" t="s">
         <v>55</v>
@@ -3161,12 +3161,12 @@
         <v>57</v>
       </c>
       <c r="M25" s="14" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>11</v>
@@ -3179,19 +3179,19 @@
         <v>P2</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F26" s="15" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G26" s="15" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H26" s="15" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I26" s="15" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="J26" s="14" t="s">
         <v>76</v>
@@ -3200,7 +3200,7 @@
         <v>56</v>
       </c>
       <c r="L26" s="15" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="M26" s="14" t="s">
         <v>83</v>
@@ -3208,7 +3208,7 @@
     </row>
     <row r="27" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B27" s="15" t="s">
         <v>11</v>
@@ -3221,19 +3221,19 @@
         <v>P3</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G27" s="15" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H27" s="15" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I27" s="15" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="J27" s="14" t="s">
         <v>55</v>
@@ -3250,7 +3250,7 @@
     </row>
     <row r="28" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>12</v>
@@ -3263,19 +3263,19 @@
         <v>P2</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F28" s="15" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="G28" s="15" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="H28" s="15" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I28" s="15" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="J28" s="14" t="s">
         <v>55</v>
@@ -3292,7 +3292,7 @@
     </row>
     <row r="29" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B29" s="15" t="s">
         <v>12</v>
@@ -3305,19 +3305,19 @@
         <v>P2</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F29" s="15" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G29" s="15" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H29" s="15" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="I29" s="15" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J29" s="14" t="s">
         <v>76</v>
@@ -3334,7 +3334,7 @@
     </row>
     <row r="30" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="14" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B30" s="15" t="s">
         <v>12</v>
@@ -3347,19 +3347,19 @@
         <v>P2</v>
       </c>
       <c r="E30" s="15" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F30" s="15" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G30" s="15" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H30" s="15" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="I30" s="15" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J30" s="14" t="s">
         <v>76</v>
@@ -3368,7 +3368,7 @@
         <v>56</v>
       </c>
       <c r="L30" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="M30" s="14" t="s">
         <v>83</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="31" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B31" s="15" t="s">
         <v>12</v>
@@ -3389,19 +3389,19 @@
         <v>P2</v>
       </c>
       <c r="E31" s="15" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F31" s="15" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="G31" s="15" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H31" s="15" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I31" s="15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J31" s="14" t="s">
         <v>55</v>
@@ -3418,7 +3418,7 @@
     </row>
     <row r="32" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="14" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>12</v>
@@ -3431,19 +3431,19 @@
         <v>P2</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F32" s="15" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G32" s="15" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H32" s="15" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I32" s="15" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J32" s="14" t="s">
         <v>55</v>
@@ -3460,7 +3460,7 @@
     </row>
     <row r="33" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B33" s="15" t="s">
         <v>12</v>
@@ -3473,19 +3473,19 @@
         <v>P3</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F33" s="15" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G33" s="15" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H33" s="15" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I33" s="15" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J33" s="14" t="s">
         <v>55</v>
@@ -3502,7 +3502,7 @@
     </row>
     <row r="34" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B34" s="15" t="s">
         <v>12</v>
@@ -3515,19 +3515,19 @@
         <v>P2</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F34" s="15" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="G34" s="15" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="H34" s="15" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="I34" s="15" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="J34" s="14" t="s">
         <v>76</v>
@@ -3536,7 +3536,7 @@
         <v>56</v>
       </c>
       <c r="L34" s="15" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="M34" s="14" t="s">
         <v>83</v>
@@ -3544,7 +3544,7 @@
     </row>
     <row r="35" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B35" s="15" t="s">
         <v>12</v>
@@ -3557,19 +3557,19 @@
         <v>P1</v>
       </c>
       <c r="E35" s="15" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F35" s="15" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="G35" s="15" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H35" s="15" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I35" s="15" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="J35" s="14" t="s">
         <v>55</v>
@@ -3578,7 +3578,7 @@
         <v>46</v>
       </c>
       <c r="L35" s="15" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="M35" s="14" t="s">
         <v>83</v>
@@ -3586,7 +3586,7 @@
     </row>
     <row r="36" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="14" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B36" s="15" t="s">
         <v>13</v>
@@ -3599,19 +3599,19 @@
         <v>P1</v>
       </c>
       <c r="E36" s="15" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F36" s="15" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="G36" s="15" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H36" s="15" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="I36" s="15" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="J36" s="14" t="s">
         <v>55</v>
@@ -3620,7 +3620,7 @@
         <v>56</v>
       </c>
       <c r="L36" s="15" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="M36" s="14" t="s">
         <v>8</v>
@@ -3628,7 +3628,7 @@
     </row>
     <row r="37" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="14" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B37" s="15" t="s">
         <v>13</v>
@@ -3641,19 +3641,19 @@
         <v>P1</v>
       </c>
       <c r="E37" s="15" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F37" s="15" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G37" s="15" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H37" s="15" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="I37" s="15" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J37" s="14" t="s">
         <v>55</v>
@@ -3670,7 +3670,7 @@
     </row>
     <row r="38" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="14" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B38" s="15" t="s">
         <v>13</v>
@@ -3683,19 +3683,19 @@
         <v>P2</v>
       </c>
       <c r="E38" s="15" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F38" s="15" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="H38" s="15" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="I38" s="15" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="J38" s="14" t="s">
         <v>55</v>
@@ -3712,7 +3712,7 @@
     </row>
     <row r="39" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="14" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B39" s="15" t="s">
         <v>13</v>
@@ -3725,19 +3725,19 @@
         <v>P2</v>
       </c>
       <c r="E39" s="15" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F39" s="15" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="H39" s="15" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="I39" s="15" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="J39" s="14" t="s">
         <v>55</v>
@@ -3754,7 +3754,7 @@
     </row>
     <row r="40" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="14" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B40" s="15" t="s">
         <v>13</v>
@@ -3767,19 +3767,19 @@
         <v>P2</v>
       </c>
       <c r="E40" s="15" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F40" s="15" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G40" s="15" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="H40" s="15" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="I40" s="15" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="J40" s="14" t="s">
         <v>55</v>
@@ -3796,7 +3796,7 @@
     </row>
     <row r="41" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B41" s="15" t="s">
         <v>13</v>
@@ -3809,19 +3809,19 @@
         <v>P2</v>
       </c>
       <c r="E41" s="15" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F41" s="15" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="H41" s="15" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="I41" s="15" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="J41" s="14" t="s">
         <v>55</v>
@@ -3838,7 +3838,7 @@
     </row>
     <row r="42" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="14" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B42" s="15" t="s">
         <v>13</v>
@@ -3851,19 +3851,19 @@
         <v>P2</v>
       </c>
       <c r="E42" s="15" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F42" s="15" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="H42" s="15" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="I42" s="15" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="J42" s="14" t="s">
         <v>55</v>
@@ -3880,7 +3880,7 @@
     </row>
     <row r="43" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B43" s="15" t="s">
         <v>13</v>
@@ -3893,19 +3893,19 @@
         <v>P2</v>
       </c>
       <c r="E43" s="15" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F43" s="15" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="H43" s="15" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="I43" s="15" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J43" s="14" t="s">
         <v>76</v>
@@ -3922,7 +3922,7 @@
     </row>
     <row r="44" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="14" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B44" s="15" t="s">
         <v>13</v>
@@ -3935,19 +3935,19 @@
         <v>P2</v>
       </c>
       <c r="E44" s="15" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F44" s="15" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="G44" s="15" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="H44" s="15" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="I44" s="15" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="J44" s="14" t="s">
         <v>55</v>
@@ -3956,7 +3956,7 @@
         <v>56</v>
       </c>
       <c r="L44" s="15" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="M44" s="14" t="s">
         <v>83</v>
@@ -3964,7 +3964,7 @@
     </row>
     <row r="45" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="14" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B45" s="15" t="s">
         <v>13</v>
@@ -3977,25 +3977,25 @@
         <v>P2</v>
       </c>
       <c r="E45" s="15" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F45" s="15" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="G45" s="15" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="H45" s="15" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="I45" s="15" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J45" s="14" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K45" s="15" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="L45" s="15" t="s">
         <v>57</v>
@@ -4006,7 +4006,7 @@
     </row>
     <row r="46" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="14" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B46" s="15" t="s">
         <v>14</v>
@@ -4019,19 +4019,19 @@
         <v>P2</v>
       </c>
       <c r="E46" s="15" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F46" s="15" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="G46" s="15" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="H46" s="15" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="I46" s="15" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="J46" s="14" t="s">
         <v>76</v>
@@ -4043,7 +4043,7 @@
         <v>57</v>
       </c>
       <c r="M46" s="14" t="s">
-        <v>321</v>
+        <v>126</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4076,7 +4076,7 @@
         <v>327</v>
       </c>
       <c r="J47" s="14" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K47" s="15" t="s">
         <v>56</v>

</xml_diff>

<commit_message>
audit F-14: surface lease-comp freshness (data-as-of + stale flag on the Lease read)
</commit_message>
<xml_diff>
--- a/docs/BSA_Application_Audit.xlsx
+++ b/docs/BSA_Application_Audit.xlsx
@@ -1949,7 +1949,7 @@
       </c>
       <c r="F7" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A7,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="F13" s="9" t="n">
         <f aca="false">SUM(F6:F12)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2867,7 +2867,7 @@
         <v>139</v>
       </c>
       <c r="M18" s="14" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
harden null-franchisor SSR crash (#329) on runs/site pages; F-45 helper dedup
</commit_message>
<xml_diff>
--- a/docs/BSA_Application_Audit.xlsx
+++ b/docs/BSA_Application_Audit.xlsx
@@ -2049,7 +2049,7 @@
       </c>
       <c r="F11" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A11,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="F13" s="9" t="n">
         <f aca="false">SUM(F6:F12)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4169,7 +4169,7 @@
         <v>57</v>
       </c>
       <c r="M49" s="14" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
security: generic intake errors, demo creds only in mock mode, rate-limit password change, IP/fail-closed/tile-cache/uuid hardening (F-24, F-27, F-28, F-29)
</commit_message>
<xml_diff>
--- a/docs/BSA_Application_Audit.xlsx
+++ b/docs/BSA_Application_Audit.xlsx
@@ -1999,7 +1999,7 @@
       </c>
       <c r="F9" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A9,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="F13" s="9" t="n">
         <f aca="false">SUM(F6:F12)</f>
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3287,7 +3287,7 @@
         <v>57</v>
       </c>
       <c r="M28" s="14" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3413,7 +3413,7 @@
         <v>57</v>
       </c>
       <c r="M31" s="14" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3455,7 +3455,7 @@
         <v>57</v>
       </c>
       <c r="M32" s="14" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3497,7 +3497,7 @@
         <v>57</v>
       </c>
       <c r="M33" s="14" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
perf/scope: White-Space reads scoped to a 15km radius around the site (F-11 local relevance, F-20 performance)
</commit_message>
<xml_diff>
--- a/docs/BSA_Application_Audit.xlsx
+++ b/docs/BSA_Application_Audit.xlsx
@@ -1949,7 +1949,7 @@
       </c>
       <c r="F7" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A7,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="F8" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A8,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="F13" s="9" t="n">
         <f aca="false">SUM(F6:F12)</f>
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2741,7 +2741,7 @@
         <v>57</v>
       </c>
       <c r="M15" s="14" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3119,7 +3119,7 @@
         <v>182</v>
       </c>
       <c r="M24" s="14" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
integrity: per-site claim to prevent concurrent double-processing (F-05); gate intake before writes + compensating rollback so failures leave no orphans (F-06)
</commit_message>
<xml_diff>
--- a/docs/BSA_Application_Audit.xlsx
+++ b/docs/BSA_Application_Audit.xlsx
@@ -276,154 +276,154 @@
     <t xml:space="preserve">lib/modules/orchestrator.ts:117-128</t>
   </si>
   <si>
+    <t xml:space="preserve">F-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A rejected or failed intake leaves orphan brands and half-written runs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For independent businesses the franchisor row is created before the 80% completeness check; intake, outlets, run and sites are then written one by one with no cleanup (no transactions on Neon HTTP).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run all validation and the completeness gate before any write; wrap the write sequence in try/catch with compensating deletes (or use a pooled client for this route).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A failed submit leaves the database unchanged; no stray brands in Franchise Screening.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">app/api/intake/route.ts:52,86,219</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Site Dashboard verdict and the Final Report recommendation can disagree for the same site.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The dashboard uses the weighted composite score (scorecard.ts: Go ≥65, Caution ≥45, Site Fit 30%, capped when Site Fit is missing). The Final Report/PDF use summariseSite, which reads only Territory, Lease and Daypart with different Daypart cut-offs (60/40).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Make one source of truth: feed the composite band into summariseSite so the recommendation can never be better than the scorecard band (or add Site Fit to summariseSite with the same weights). Add a unit test asserting the two always agree.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A broker sees the same Proceed / Caution / No-Go call on the dashboard, the Final Report and the PDF.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/modules/scorecard.ts:40-42,102; lib/modules/siteVerdict.ts:87-144</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincial lease reads use an NCR-only rent-to-land calibration and NCR wording.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The ₱6–14 per ₱1,000 zonal band and the "typical NCR band" text were calibrated on NCR corridors but are applied to Davao, Cavite and Batangas zonal values.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Store a calibration band per region in the region registry; return 'unknown' and hide the cross-check when a region has none; make the note text region-aware.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincial rent-to-land cross-checks are either calibrated for that region or honestly withheld.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/modules/leaseMath.ts:272-331; lib/modules/leaseBenchmark.ts:180-182</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Several code paths still silently default to NCR.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lease falls back to the Quezon City corridor for any region; zonal lookups default to 'NCR'; ingest sweeps default to the NCR grid.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resolve the fallback corridor per region from the registry; return null / 'no data' when a region has no zonal rows; require --region on ingest scripts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A Cavite or Batangas site is never scored against Metro Manila data without a clear flag.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/modules/orchestrator.ts:55,176; lib/modules/p2p3Modules.ts:282; lib/modules/leaseBenchmark.ts:62; lib/geo/zonalRow.ts:39; lib/ingest/places.ts:231,324,403,461</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Some modules report a value when they actually have no data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daypart's last-resort nearest demographic cell has no distance cap (can borrow another region's cell); a silently failed OSM warm returns 0 competitors, so Informal scores a perfect 100; Healthcare uses cnt ?? 0.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cap the nearest-cell fallback (e.g. 5 km); propagate a 'coverage unknown' flag from the POI cache and return null scores when coverage failed; treat missing counts as null, not 0.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missing data shows as "—" / low confidence, never as a strong score (Truth Layer rule).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/modules/p2p3Modules.ts:66-70,142,173; lib/places/poiCache.ts:129,186</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">White-Space can recommend barangays in another region (e.g. Davao areas for an NCR site).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The White-Space ranking has no region or distance limit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filter candidate areas by the site's region and a maximum distance (e.g. ST_DWithin 10–15 km).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">White-Space suggestions are always local and actionable for the broker.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/modules/p2p3Math.ts:387-389</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The schema allows duplicate or colliding reference data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mall_property has no unique key but is upserted by mall name (same-name malls in different regions overwrite each other); lease_comp has no natural key; demographic_cell has no region column.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add region to mall_property + unique (region, mall_name); add a natural key to lease_comp; add region to demographic_cell (backfill from admin_boundary); update the loaders.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loading one province can never overwrite another's malls or comps; region-scoped reads become cheap.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prisma/schema.prisma:398-457; lib/ingest/loaders.ts:185</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In progress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A failed lease load can wipe a corridor's comps.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">loadLease deletes each (format, corridor) group and re-inserts it without a transaction.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insert the new rows first, then delete the old rows by id (or load through a pooled client inside a transaction).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Re-loading comps is always safe; a corridor is never left empty.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/ingest/loaders.ts:112-133</t>
+  </si>
+  <si>
     <t xml:space="preserve">Open</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A rejected or failed intake leaves orphan brands and half-written runs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">For independent businesses the franchisor row is created before the 80% completeness check; intake, outlets, run and sites are then written one by one with no cleanup (no transactions on Neon HTTP).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Run all validation and the completeness gate before any write; wrap the write sequence in try/catch with compensating deletes (or use a pooled client for this route).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A failed submit leaves the database unchanged; no stray brands in Franchise Screening.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">app/api/intake/route.ts:52,86,219</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Site Dashboard verdict and the Final Report recommendation can disagree for the same site.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The dashboard uses the weighted composite score (scorecard.ts: Go ≥65, Caution ≥45, Site Fit 30%, capped when Site Fit is missing). The Final Report/PDF use summariseSite, which reads only Territory, Lease and Daypart with different Daypart cut-offs (60/40).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Make one source of truth: feed the composite band into summariseSite so the recommendation can never be better than the scorecard band (or add Site Fit to summariseSite with the same weights). Add a unit test asserting the two always agree.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A broker sees the same Proceed / Caution / No-Go call on the dashboard, the Final Report and the PDF.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/modules/scorecard.ts:40-42,102; lib/modules/siteVerdict.ts:87-144</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Provincial lease reads use an NCR-only rent-to-land calibration and NCR wording.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The ₱6–14 per ₱1,000 zonal band and the "typical NCR band" text were calibrated on NCR corridors but are applied to Davao, Cavite and Batangas zonal values.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Store a calibration band per region in the region registry; return 'unknown' and hide the cross-check when a region has none; make the note text region-aware.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Provincial rent-to-land cross-checks are either calibrated for that region or honestly withheld.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/modules/leaseMath.ts:272-331; lib/modules/leaseBenchmark.ts:180-182</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Several code paths still silently default to NCR.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lease falls back to the Quezon City corridor for any region; zonal lookups default to 'NCR'; ingest sweeps default to the NCR grid.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resolve the fallback corridor per region from the registry; return null / 'no data' when a region has no zonal rows; require --region on ingest scripts.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A Cavite or Batangas site is never scored against Metro Manila data without a clear flag.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/modules/orchestrator.ts:55,176; lib/modules/p2p3Modules.ts:282; lib/modules/leaseBenchmark.ts:62; lib/geo/zonalRow.ts:39; lib/ingest/places.ts:231,324,403,461</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Some modules report a value when they actually have no data.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Daypart's last-resort nearest demographic cell has no distance cap (can borrow another region's cell); a silently failed OSM warm returns 0 competitors, so Informal scores a perfect 100; Healthcare uses cnt ?? 0.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cap the nearest-cell fallback (e.g. 5 km); propagate a 'coverage unknown' flag from the POI cache and return null scores when coverage failed; treat missing counts as null, not 0.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Missing data shows as "—" / low confidence, never as a strong score (Truth Layer rule).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/modules/p2p3Modules.ts:66-70,142,173; lib/places/poiCache.ts:129,186</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">White-Space can recommend barangays in another region (e.g. Davao areas for an NCR site).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The White-Space ranking has no region or distance limit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Filter candidate areas by the site's region and a maximum distance (e.g. ST_DWithin 10–15 km).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">White-Space suggestions are always local and actionable for the broker.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/modules/p2p3Math.ts:387-389</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The schema allows duplicate or colliding reference data.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mall_property has no unique key but is upserted by mall name (same-name malls in different regions overwrite each other); lease_comp has no natural key; demographic_cell has no region column.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add region to mall_property + unique (region, mall_name); add a natural key to lease_comp; add region to demographic_cell (backfill from admin_boundary); update the loaders.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loading one province can never overwrite another's malls or comps; region-scoped reads become cheap.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prisma/schema.prisma:398-457; lib/ingest/loaders.ts:185</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In progress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A failed lease load can wipe a corridor's comps.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">loadLease deletes each (format, corridor) group and re-inserts it without a transaction.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Insert the new rows first, then delete the old rows by id (or load through a pooled client inside a transaction).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Re-loading comps is always safe; a corridor is never left empty.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/ingest/loaders.ts:112-133</t>
   </si>
   <si>
     <t xml:space="preserve">F-14</t>
@@ -1924,7 +1924,7 @@
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A6,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="F13" s="9" t="n">
         <f aca="false">SUM(F6:F12)</f>
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2489,12 +2489,12 @@
         <v>57</v>
       </c>
       <c r="M9" s="14" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>9</v>
@@ -2507,19 +2507,19 @@
         <v>P2</v>
       </c>
       <c r="E10" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="F10" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="G10" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="G10" s="15" t="s">
+      <c r="H10" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="H10" s="15" t="s">
+      <c r="I10" s="15" t="s">
         <v>88</v>
-      </c>
-      <c r="I10" s="15" t="s">
-        <v>89</v>
       </c>
       <c r="J10" s="14" t="s">
         <v>76</v>
@@ -2531,12 +2531,12 @@
         <v>57</v>
       </c>
       <c r="M10" s="14" t="s">
-        <v>83</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>10</v>
@@ -2549,19 +2549,19 @@
         <v>P1</v>
       </c>
       <c r="E11" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="F11" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="G11" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="G11" s="15" t="s">
+      <c r="H11" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="H11" s="15" t="s">
+      <c r="I11" s="15" t="s">
         <v>94</v>
-      </c>
-      <c r="I11" s="15" t="s">
-        <v>95</v>
       </c>
       <c r="J11" s="14" t="s">
         <v>76</v>
@@ -2578,7 +2578,7 @@
     </row>
     <row r="12" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B12" s="15" t="s">
         <v>10</v>
@@ -2591,19 +2591,19 @@
         <v>P1</v>
       </c>
       <c r="E12" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="F12" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="G12" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="G12" s="15" t="s">
+      <c r="H12" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="H12" s="15" t="s">
+      <c r="I12" s="15" t="s">
         <v>100</v>
-      </c>
-      <c r="I12" s="15" t="s">
-        <v>101</v>
       </c>
       <c r="J12" s="14" t="s">
         <v>76</v>
@@ -2620,7 +2620,7 @@
     </row>
     <row r="13" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B13" s="15" t="s">
         <v>10</v>
@@ -2633,19 +2633,19 @@
         <v>P2</v>
       </c>
       <c r="E13" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="F13" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="G13" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="G13" s="15" t="s">
+      <c r="H13" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="H13" s="15" t="s">
+      <c r="I13" s="15" t="s">
         <v>106</v>
-      </c>
-      <c r="I13" s="15" t="s">
-        <v>107</v>
       </c>
       <c r="J13" s="14" t="s">
         <v>76</v>
@@ -2662,7 +2662,7 @@
     </row>
     <row r="14" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B14" s="15" t="s">
         <v>10</v>
@@ -2675,19 +2675,19 @@
         <v>P2</v>
       </c>
       <c r="E14" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="F14" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="F14" s="15" t="s">
+      <c r="G14" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="G14" s="15" t="s">
+      <c r="H14" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="H14" s="15" t="s">
+      <c r="I14" s="15" t="s">
         <v>112</v>
-      </c>
-      <c r="I14" s="15" t="s">
-        <v>113</v>
       </c>
       <c r="J14" s="14" t="s">
         <v>76</v>
@@ -2704,7 +2704,7 @@
     </row>
     <row r="15" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B15" s="15" t="s">
         <v>10</v>
@@ -2717,19 +2717,19 @@
         <v>P2</v>
       </c>
       <c r="E15" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="F15" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="F15" s="15" t="s">
+      <c r="G15" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="G15" s="15" t="s">
+      <c r="H15" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="H15" s="15" t="s">
+      <c r="I15" s="15" t="s">
         <v>118</v>
-      </c>
-      <c r="I15" s="15" t="s">
-        <v>119</v>
       </c>
       <c r="J15" s="14" t="s">
         <v>55</v>
@@ -2746,7 +2746,7 @@
     </row>
     <row r="16" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B16" s="15" t="s">
         <v>10</v>
@@ -2759,19 +2759,19 @@
         <v>P2</v>
       </c>
       <c r="E16" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="F16" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="F16" s="15" t="s">
+      <c r="G16" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="G16" s="15" t="s">
+      <c r="H16" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="H16" s="15" t="s">
+      <c r="I16" s="15" t="s">
         <v>124</v>
-      </c>
-      <c r="I16" s="15" t="s">
-        <v>125</v>
       </c>
       <c r="J16" s="14" t="s">
         <v>76</v>
@@ -2783,12 +2783,12 @@
         <v>57</v>
       </c>
       <c r="M16" s="14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B17" s="15" t="s">
         <v>10</v>
@@ -2801,19 +2801,19 @@
         <v>P2</v>
       </c>
       <c r="E17" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="F17" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="F17" s="15" t="s">
+      <c r="G17" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="G17" s="15" t="s">
+      <c r="H17" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="H17" s="15" t="s">
+      <c r="I17" s="15" t="s">
         <v>131</v>
-      </c>
-      <c r="I17" s="15" t="s">
-        <v>132</v>
       </c>
       <c r="J17" s="14" t="s">
         <v>55</v>
@@ -2825,7 +2825,7 @@
         <v>57</v>
       </c>
       <c r="M17" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2909,7 +2909,7 @@
         <v>146</v>
       </c>
       <c r="M19" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2951,7 +2951,7 @@
         <v>154</v>
       </c>
       <c r="M20" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2993,7 +2993,7 @@
         <v>161</v>
       </c>
       <c r="M21" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3035,7 +3035,7 @@
         <v>168</v>
       </c>
       <c r="M22" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3077,7 +3077,7 @@
         <v>175</v>
       </c>
       <c r="M23" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3203,7 +3203,7 @@
         <v>195</v>
       </c>
       <c r="M26" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3245,7 +3245,7 @@
         <v>57</v>
       </c>
       <c r="M27" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3329,7 +3329,7 @@
         <v>57</v>
       </c>
       <c r="M29" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3371,7 +3371,7 @@
         <v>220</v>
       </c>
       <c r="M30" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3539,7 +3539,7 @@
         <v>245</v>
       </c>
       <c r="M34" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3581,7 +3581,7 @@
         <v>252</v>
       </c>
       <c r="M35" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3791,7 +3791,7 @@
         <v>57</v>
       </c>
       <c r="M40" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3833,7 +3833,7 @@
         <v>57</v>
       </c>
       <c r="M41" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3917,7 +3917,7 @@
         <v>57</v>
       </c>
       <c r="M43" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3959,7 +3959,7 @@
         <v>308</v>
       </c>
       <c r="M44" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4001,7 +4001,7 @@
         <v>57</v>
       </c>
       <c r="M45" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4043,7 +4043,7 @@
         <v>57</v>
       </c>
       <c r="M46" s="14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4085,7 +4085,7 @@
         <v>328</v>
       </c>
       <c r="M47" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4127,7 +4127,7 @@
         <v>57</v>
       </c>
       <c r="M48" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4211,7 +4211,7 @@
         <v>347</v>
       </c>
       <c r="M50" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4253,7 +4253,7 @@
         <v>354</v>
       </c>
       <c r="M51" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4421,7 +4421,7 @@
         <v>382</v>
       </c>
       <c r="M55" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4463,7 +4463,7 @@
         <v>57</v>
       </c>
       <c r="M56" s="14" t="s">
-        <v>83</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
perf: batch POI/demographic loaders via direct pooled client (F-22); single-scan + 5-min cache for /api/brands (F-23)
</commit_message>
<xml_diff>
--- a/docs/BSA_Application_Audit.xlsx
+++ b/docs/BSA_Application_Audit.xlsx
@@ -1949,7 +1949,7 @@
       </c>
       <c r="F7" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A7,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="F8" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A8,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="F13" s="9" t="n">
         <f aca="false">SUM(F6:F12)</f>
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2909,7 +2909,7 @@
         <v>146</v>
       </c>
       <c r="M19" s="14" t="s">
-        <v>132</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3035,7 +3035,7 @@
         <v>168</v>
       </c>
       <c r="M22" s="14" t="s">
-        <v>132</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3203,7 +3203,7 @@
         <v>195</v>
       </c>
       <c r="M26" s="14" t="s">
-        <v>132</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3245,7 +3245,7 @@
         <v>57</v>
       </c>
       <c r="M27" s="14" t="s">
-        <v>132</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
ux/a11y: aria-labels on intake inputs + icon buttons (F-36); responsive intake rows + scrollable lease table (F-37); 12px text floor (F-39); lease corridor picker to fix a proxy benchmark (F-40)
</commit_message>
<xml_diff>
--- a/docs/BSA_Application_Audit.xlsx
+++ b/docs/BSA_Application_Audit.xlsx
@@ -2024,7 +2024,7 @@
       </c>
       <c r="F10" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A10,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="F13" s="9" t="n">
         <f aca="false">SUM(F6:F12)</f>
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3791,7 +3791,7 @@
         <v>57</v>
       </c>
       <c r="M40" s="14" t="s">
-        <v>132</v>
+        <v>8</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3833,7 +3833,7 @@
         <v>57</v>
       </c>
       <c r="M41" s="14" t="s">
-        <v>132</v>
+        <v>8</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3917,7 +3917,7 @@
         <v>57</v>
       </c>
       <c r="M43" s="14" t="s">
-        <v>132</v>
+        <v>8</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3959,7 +3959,7 @@
         <v>308</v>
       </c>
       <c r="M44" s="14" t="s">
-        <v>132</v>
+        <v>8</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4001,7 +4001,7 @@
         <v>57</v>
       </c>
       <c r="M45" s="14" t="s">
-        <v>132</v>
+        <v>8</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
refactor: service layer for runs/sites/reports/account so pages stop reading Prisma directly (F-47); type PDF element + document reserved enum values (F-46); status corrections
</commit_message>
<xml_diff>
--- a/docs/BSA_Application_Audit.xlsx
+++ b/docs/BSA_Application_Audit.xlsx
@@ -402,616 +402,616 @@
     <t xml:space="preserve">prisma/schema.prisma:398-457; lib/ingest/loaders.ts:185</t>
   </si>
   <si>
+    <t xml:space="preserve">F-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A failed lease load can wipe a corridor's comps.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">loadLease deletes each (format, corridor) group and re-inserts it without a transaction.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insert the new rows first, then delete the old rows by id (or load through a pooled client inside a transaction).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Re-loading comps is always safe; a corridor is never left empty.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/ingest/loaders.ts:112-133</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lease comps have no freshness rule.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">observedDate is only used for ordering; old comps are never flagged or aged out.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flag comps older than 18 months, down-weight or exclude them past 36 months, and show 'data as of' on the Lease tab. Optional broker endpoint to submit confirmed rents.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rent benchmarks reflect the current market and say how recent they are.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/modules/leaseBenchmark.ts:122-153</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior backlog D-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Site Fit 'accessibility' pillar is always empty.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No transport layer is loaded, so the 15% accessibility pillar is null for every site.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load OSM transport features (jeepney/bus stops, rail stations, major roads) per region and score distance/density to them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site Fit reflects how easy a site is to reach — important for Filipino commuter traffic.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/modules/siteFit.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior backlog D-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trade areas are fixed circles.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catchments are circles by format (600–1,200 m); rivers, highways and gated areas are ignored.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use travel-time isochrones (self-hosted OSRM/Valhalla or an isochrone API), cached per site.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catchments match how customers actually reach the site.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/modules/territoryMath.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior backlog D-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Known NCR zonal gaps (San Juan missing, Valenzuela barangay grain).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The BIR workbooks for those RDOs were never loaded.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Download the current schedules and load them with npm run db:load-zonal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The zonal cross-check works for every NCR city.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prisma/data/zonal/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior backlog D-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google-sourced POIs are recorded as 'manual'; age profiles are modelled from income; old runs keep pre-fix scores.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PoiSource enum has no 'google'; age_profile is a Projected model; historical runs were never re-run after the fix batches.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add 'google' to PoiSource plus a provenance column; load PSA age-sex tables; run a one-off re-run script for historical runs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clean provenance, real age data, and consistent scores across all runs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prisma/schema.prisma; prisma/enrichAgeProfiles.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior backlog D-05/06/07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cavite and Batangas are wired in code but have no reference data loaded yet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The R-series built the loaders; the owner data loads (boundaries, OSM sweep, PSA population, BIR zonal, lease comps, malls, traffic AADT) have not been run.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Follow the one-province load order in docs/qa-history/QA_JOURNEY_FINDINGS_CALABARZON.md (boundaries → OSM ingest in a quiet window → demographics → zonal → lease → malls → traffic), then re-run a Cavite and a Batangas intake.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincial sites get real scores instead of 'no data' / Projected fallbacks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/qa-history/QA_JOURNEY_FINDINGS_CALABARZON.md; prisma/data/*/README.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R-series follow-up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">White-Space loads every competitor POI and every demographic cell for each site.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No region/bbox filter on the reads; scoring is an in-memory areas × POIs loop in JavaScript.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Push the counting into PostGIS (ST_DWithin + GROUP BY area) scoped to the site's region/radius; compute once per run and cache by (run, concept).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">White-Space runs in well under a second and keeps scaling as provinces are added.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/modules/p2p3Modules.ts:381-497</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New audit / Prior A-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missing and inefficient database indexes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No index on module_result.pipeline_run_id (filtered on every dashboard load and cascade delete); nearest-row lookups ORDER BY ST_Distance (full scan) instead of the KNN &lt;-&gt; operator; duplicate GiST index on demographic_cell.geom; migration_lock.toml missing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add @@index([pipelineRunId]) to ModuleResult; rewrite nearest lookups with ORDER BY geom &lt;-&gt; point; drop the duplicate GiST index; commit migration_lock.toml.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faster dashboards and module reads; a clean migration history.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prisma/schema.prisma:518-534; lib/modules/p2p3Modules.ts:69,189; prisma/migrations/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference-data loaders write one row at a time over Neon HTTP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loaders do find-then-write per row (2–3 round trips each), so a province-scale load is very slow.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Batch INSERT … ON CONFLICT in chunks of about 500 using a script-only client on the direct (pooled) connection.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Province loads finish in minutes, not hours.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/ingest/loaders.ts:55-63,185-192,216-230</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior backlog A-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/api/brands runs a full ILIKE scan of the POI table per catalog brand on every call.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No caching; the per-brand scans run one after another.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precompute branch counts (materialised view or nightly job) or cache the response.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Franchise Screening loads instantly.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">app/api/brands/route.ts:21-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The intake route can leak raw database error text to the browser.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The 500 response includes err.message; Prisma/Neon messages can contain query and column details.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log the full error server-side; return a generic message plus a short reason code.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No internal details reach the client (passes a basic pen-test check).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">app/api/intake/route.ts:219-220</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nothing limits calls to paid Google APIs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any signed-in user (and registration is open) can call /api/places, /api/geocode and /api/maptiles; lat/lon/types/address inputs have loose bounds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add per-user daily quotas (reuse the DB rate limiter), tighten Zod bounds (PH bounding box, max lengths), and consider invite-only registration.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Predictable Google API cost; no abuse through the proxy routes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">app/api/places/route.ts:11-25; app/api/geocode/route.ts:7-13; app/api/maptiles/route.ts:12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sessions can't be revoked, and role changes don't take effect until the token expires.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stateless 8-hour JWTs; logout only clears the cookie; role and franchisor are read from the token, not the database.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add token_version (or sessions_valid_after) to app_user; bump it on logout-all, password change and role change; check it in getSession.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logging out, changing a password or demoting a user takes effect immediately.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/auth/auth.ts:42-64; app/api/auth/logout/route.ts:6; app/api/auth/password/route.ts:43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New audit / Prior S-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The login page ships prefilled with demo credentials on production.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Default email/password state and a demo hint are hard-coded in the login page, even though demo logins are refused on deployments.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Render the defaults and the hint only when mock auth is enabled (pass a server flag to the page).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Production users see a clean login with no dead or sensitive-looking credentials.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">app/(auth)/login/page.tsx:12-13,76</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The password-change route has no rate limit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A hijacked session could brute-force the current password.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apply the existing checkLimit to /api/auth/password.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Password change is protected like login.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">app/api/auth/password/route.ts:36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Several small hardening gaps.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Territory Guard has no isUuid guard (malformed ids return 500); authenticated map tiles are sent Cache-Control: public; the login IP limiter trusts x-forwarded-for off Netlify and fails open on DB errors; the user's email is written into brand 'positioning' text.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add the isUuid guard; switch tiles to private caching; trust only the platform client-IP header and fail closed; stop writing the email into brand text.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clean results on the low-severity pen-test checks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">app/api/territory-guard/route.ts:33; app/api/maptiles/[z]/[x]/[y]/route.ts:36; lib/auth/rateLimit.ts:37-52; app/api/franchisors/route.ts:103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The CSP still allows inline scripts and there is no central route guard.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Next 14 bootstrap needs 'unsafe-inline' without nonces; there is no middleware.ts, so every new route must remember its own auth check.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add middleware.ts that generates a per-request nonce for a strict CSP and redirects unauthenticated requests for app pages and APIs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stronger XSS protection, and auth that can't be forgotten on a new route.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">next.config.mjs:36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior backlog S-02/S-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exposed credentials still need rotating.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A Google API key was exposed in keys.docx and real account passwords were in an old database dump (repo history since cleaned).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rotate the Google key (restrict by API + referrer) and reset the affected passwords; confirm the repo is private.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No credential that was ever exposed remains valid.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Owner action (Google Cloud console, Netlify env)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior backlog S-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">There is no navigation on phones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Below the md breakpoint the sidebar is hidden; the mobile top bar only has the logo and Logout.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add a hamburger drawer (or bottom tab bar) that renders the same SidebarNav items plus Settings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brokers in the field can reach Franchise Screening, New Intake and Settings from a phone.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">app/(app)/layout.tsx:34,59-64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New audit / Prior U-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The first-run tour points at menu items that no longer exist.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tour steps still target nav-modules and nav-reports and describe removed screens; anchored steps also miss on mobile.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rewrite the tour for the current menu (Franchise Screening → New Intake → Site Dashboard → Final Report/PDF); skip or re-anchor steps on mobile.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New users get an accurate guided tour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">components/OnboardingTour.tsx:30-58,91-92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Removed pages are still linked or reachable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/reports is linked from the dashboard; /explore, /modules and /scorecard still build and load by URL (Scorecard badges also fail contrast: white text on green/amber).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decide per page: remove the page and its components (ModulesView, PlacesExplorer, ReportView, PrintButton) with redirects, or keep and fix it. Update the RunDashboard links.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No dead-end or off-brand screens, and a smaller codebase for handoff.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">components/RunDashboard.tsx:69; app/(app)/{explore,modules,scorecard,reports}/page.tsx; app/(app)/scorecard/page.tsx:19-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keyboard and screen-reader users can't use the site tabs properly, and focus is invisible.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabs are plain buttons with no tab roles, aria-selected or arrow keys; there are no focus-visible styles anywhere and .field removes the outline.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add role=tablist/tab/tabpanel, aria-selected and arrow-key handling; add focus-visible:ring-2 ring-accent to buttons, nav items and fields.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WCAG 2.2 AA keyboard and focus compliance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">components/SiteIntelligenceTabs.tsx:204-217; app/globals.css:52-61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Some inputs and icon buttons have no accessible label.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intake outlet/candidate rows rely on placeholders; the location picker search and its ✕ close button have no labels.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add visible labels or aria-labels to every input and icon button.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forms work with screen readers and are clearer for older users.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">components/SteppedIntakeWizard.tsx:675-702; components/LocationPicker.tsx:131-134</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Layouts overflow on small screens.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intake rows use a fixed grid-cols-12; the lease comps table is overflow-hidden.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use grid-cols-1 sm:grid-cols-12 for the rows; switch the table wrapper to overflow-x-auto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The intake and the Lease tab work on phones and small laptops.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">components/SteppedIntakeWizard.tsx:674,699; components/SiteIntelligenceTabs.tsx:510</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">There are no branded loading, error or not-found screens.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No loading.tsx / error.tsx / not-found.tsx files exist, so failures show the default Next.js page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add them under app/(app)/ in the GRID theme, with a retry action and plain-language copy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Errors are calm, branded and recoverable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">app/(app)/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very small text is used widely (9–11px).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">63 uses of text-[9–11px], often in muted grey — hard to read for older users.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set a 12px minimum (13–14px for body copy); raise muted-text contrast where it sits on hover surfaces.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Readable for the older / tech-resistant audience named in the brand guidelines.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">components/SiteIntelligenceTabs.tsx; components/SteppedIntakeWizard.tsx:601</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The proxy lease corridor can't be corrected, and the map ring colour can lag the verdict.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When no corridor matches, the Lease tab says it's a proxy but offers no picker; TerritoryMap computes its own verdict.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add a corridor picker (corridorsForRegion + corridors that have comps) that re-benchmarks; pass the blended verdict into TerritoryMap.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brokers can fix the corridor in one click, and the map always matches the verdict.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">components/SiteIntelligenceTabs.tsx; components/TerritoryMap.tsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior backlog U-02/U-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The UI redesign has not been done yet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branding (palette, fonts, logo) is applied, but hierarchy, spacing and components were never designed as a system.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run docs/DESIGN_PROMPT.md in a Claude design session, then implement the resulting tokens and component recipes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A cohesive, professional UI where the Proceed / Caution / No-Go call is obvious in under 5 seconds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/DESIGN_PROMPT.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Owner + Dev team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leftover AI code, config and docs remain after the AI report was removed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/ai/index.ts still lists 'vectorshift'; analysisCache/mockAnalysis/outputCheck/analysisPrompts are only used by tests; the orchestrator still deletes module='analysis' rows and site/page reads them; the PipelineUsage model remains; .env.example keeps a VectorShift section (with a real-looking pipeline id); generateGrounded writes placeholder aiGeneration rows; UI copy still says 'write-up'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove the unused lib/ai files and their tests; drop the vectorshift provider option; remove the 'analysis' reads/deletes; drop PipelineUsage/AiGeneration via migration (or mark them reserved); clean .env.example and UI copy; remove VECTORSHIFT_* / ANALYSIS_BACKGROUND / INTERNAL_JOB_SECRET from Netlify.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A codebase that matches the product, with no dead AI paths for the dev team to puzzle over.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/ai/*; lib/modules/orchestrator.ts:8,113; app/(app)/site/page.tsx:66; prisma/schema.prisma:592-620; .env.example</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Critical server modules have no tests.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tests cover pure math only: nothing tests orchestrator slicing/resume/failure, p2p3Modules (White-Space scope, fallbacks), territoryGuard, leaseBenchmark zonal resolution, siteFit, poiCache or the loaders; no test checks that summariseSite agrees with the scorecard; no end-to-end journey test.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add integration tests against a Neon test branch (or local Postgres + PostGIS in CI); add the verdict-agreement test; add Playwright smoke tests (login → intake → run → site tabs → PDF).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regressions are caught before deploy, and the handoff is backed by tests.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/unit; lib/modules/*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New audit / Prior A-04</t>
+  </si>
+  <si>
     <t xml:space="preserve">In progress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A failed lease load can wipe a corridor's comps.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">loadLease deletes each (format, corridor) group and re-inserts it without a transaction.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Insert the new rows first, then delete the old rows by id (or load through a pooled client inside a transaction).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Re-loading comps is always safe; a corridor is never left empty.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/ingest/loaders.ts:112-133</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lease comps have no freshness rule.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">observedDate is only used for ordering; old comps are never flagged or aged out.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flag comps older than 18 months, down-weight or exclude them past 36 months, and show 'data as of' on the Lease tab. Optional broker endpoint to submit confirmed rents.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rent benchmarks reflect the current market and say how recent they are.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/modules/leaseBenchmark.ts:122-153</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prior backlog D-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Site Fit 'accessibility' pillar is always empty.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No transport layer is loaded, so the 15% accessibility pillar is null for every site.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Load OSM transport features (jeepney/bus stops, rail stations, major roads) per region and score distance/density to them.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Site Fit reflects how easy a site is to reach — important for Filipino commuter traffic.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/modules/siteFit.ts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prior backlog D-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trade areas are fixed circles.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Catchments are circles by format (600–1,200 m); rivers, highways and gated areas are ignored.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use travel-time isochrones (self-hosted OSRM/Valhalla or an isochrone API), cached per site.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Catchments match how customers actually reach the site.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/modules/territoryMath.ts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prior backlog D-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Known NCR zonal gaps (San Juan missing, Valenzuela barangay grain).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The BIR workbooks for those RDOs were never loaded.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Download the current schedules and load them with npm run db:load-zonal.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The zonal cross-check works for every NCR city.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prisma/data/zonal/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prior backlog D-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Google-sourced POIs are recorded as 'manual'; age profiles are modelled from income; old runs keep pre-fix scores.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PoiSource enum has no 'google'; age_profile is a Projected model; historical runs were never re-run after the fix batches.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add 'google' to PoiSource plus a provenance column; load PSA age-sex tables; run a one-off re-run script for historical runs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clean provenance, real age data, and consistent scores across all runs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prisma/schema.prisma; prisma/enrichAgeProfiles.ts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prior backlog D-05/06/07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cavite and Batangas are wired in code but have no reference data loaded yet.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The R-series built the loaders; the owner data loads (boundaries, OSM sweep, PSA population, BIR zonal, lease comps, malls, traffic AADT) have not been run.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Follow the one-province load order in docs/qa-history/QA_JOURNEY_FINDINGS_CALABARZON.md (boundaries → OSM ingest in a quiet window → demographics → zonal → lease → malls → traffic), then re-run a Cavite and a Batangas intake.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Provincial sites get real scores instead of 'no data' / Projected fallbacks.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/qa-history/QA_JOURNEY_FINDINGS_CALABARZON.md; prisma/data/*/README.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R-series follow-up</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">White-Space loads every competitor POI and every demographic cell for each site.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No region/bbox filter on the reads; scoring is an in-memory areas × POIs loop in JavaScript.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Push the counting into PostGIS (ST_DWithin + GROUP BY area) scoped to the site's region/radius; compute once per run and cache by (run, concept).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">White-Space runs in well under a second and keeps scaling as provinces are added.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/modules/p2p3Modules.ts:381-497</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New audit / Prior A-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Missing and inefficient database indexes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No index on module_result.pipeline_run_id (filtered on every dashboard load and cascade delete); nearest-row lookups ORDER BY ST_Distance (full scan) instead of the KNN &lt;-&gt; operator; duplicate GiST index on demographic_cell.geom; migration_lock.toml missing.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add @@index([pipelineRunId]) to ModuleResult; rewrite nearest lookups with ORDER BY geom &lt;-&gt; point; drop the duplicate GiST index; commit migration_lock.toml.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Faster dashboards and module reads; a clean migration history.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prisma/schema.prisma:518-534; lib/modules/p2p3Modules.ts:69,189; prisma/migrations/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reference-data loaders write one row at a time over Neon HTTP.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loaders do find-then-write per row (2–3 round trips each), so a province-scale load is very slow.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Batch INSERT … ON CONFLICT in chunks of about 500 using a script-only client on the direct (pooled) connection.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Province loads finish in minutes, not hours.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/ingest/loaders.ts:55-63,185-192,216-230</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prior backlog A-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/api/brands runs a full ILIKE scan of the POI table per catalog brand on every call.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No caching; the per-brand scans run one after another.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Precompute branch counts (materialised view or nightly job) or cache the response.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Franchise Screening loads instantly.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">app/api/brands/route.ts:21-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The intake route can leak raw database error text to the browser.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The 500 response includes err.message; Prisma/Neon messages can contain query and column details.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Log the full error server-side; return a generic message plus a short reason code.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No internal details reach the client (passes a basic pen-test check).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">app/api/intake/route.ts:219-220</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nothing limits calls to paid Google APIs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Any signed-in user (and registration is open) can call /api/places, /api/geocode and /api/maptiles; lat/lon/types/address inputs have loose bounds.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add per-user daily quotas (reuse the DB rate limiter), tighten Zod bounds (PH bounding box, max lengths), and consider invite-only registration.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Predictable Google API cost; no abuse through the proxy routes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">app/api/places/route.ts:11-25; app/api/geocode/route.ts:7-13; app/api/maptiles/route.ts:12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sessions can't be revoked, and role changes don't take effect until the token expires.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stateless 8-hour JWTs; logout only clears the cookie; role and franchisor are read from the token, not the database.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add token_version (or sessions_valid_after) to app_user; bump it on logout-all, password change and role change; check it in getSession.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Logging out, changing a password or demoting a user takes effect immediately.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/auth/auth.ts:42-64; app/api/auth/logout/route.ts:6; app/api/auth/password/route.ts:43</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New audit / Prior S-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The login page ships prefilled with demo credentials on production.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Default email/password state and a demo hint are hard-coded in the login page, even though demo logins are refused on deployments.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Render the defaults and the hint only when mock auth is enabled (pass a server flag to the page).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Production users see a clean login with no dead or sensitive-looking credentials.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">app/(auth)/login/page.tsx:12-13,76</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The password-change route has no rate limit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A hijacked session could brute-force the current password.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apply the existing checkLimit to /api/auth/password.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Password change is protected like login.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">app/api/auth/password/route.ts:36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Several small hardening gaps.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Territory Guard has no isUuid guard (malformed ids return 500); authenticated map tiles are sent Cache-Control: public; the login IP limiter trusts x-forwarded-for off Netlify and fails open on DB errors; the user's email is written into brand 'positioning' text.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add the isUuid guard; switch tiles to private caching; trust only the platform client-IP header and fail closed; stop writing the email into brand text.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clean results on the low-severity pen-test checks.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">app/api/territory-guard/route.ts:33; app/api/maptiles/[z]/[x]/[y]/route.ts:36; lib/auth/rateLimit.ts:37-52; app/api/franchisors/route.ts:103</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The CSP still allows inline scripts and there is no central route guard.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Next 14 bootstrap needs 'unsafe-inline' without nonces; there is no middleware.ts, so every new route must remember its own auth check.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add middleware.ts that generates a per-request nonce for a strict CSP and redirects unauthenticated requests for app pages and APIs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stronger XSS protection, and auth that can't be forgotten on a new route.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">next.config.mjs:36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prior backlog S-02/S-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exposed credentials still need rotating.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A Google API key was exposed in keys.docx and real account passwords were in an old database dump (repo history since cleaned).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rotate the Google key (restrict by API + referrer) and reset the affected passwords; confirm the repo is private.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No credential that was ever exposed remains valid.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Owner action (Google Cloud console, Netlify env)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prior backlog S-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">There is no navigation on phones.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Below the md breakpoint the sidebar is hidden; the mobile top bar only has the logo and Logout.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add a hamburger drawer (or bottom tab bar) that renders the same SidebarNav items plus Settings.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brokers in the field can reach Franchise Screening, New Intake and Settings from a phone.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">app/(app)/layout.tsx:34,59-64</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New audit / Prior U-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-33</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The first-run tour points at menu items that no longer exist.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tour steps still target nav-modules and nav-reports and describe removed screens; anchored steps also miss on mobile.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rewrite the tour for the current menu (Franchise Screening → New Intake → Site Dashboard → Final Report/PDF); skip or re-anchor steps on mobile.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New users get an accurate guided tour.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">components/OnboardingTour.tsx:30-58,91-92</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-34</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Removed pages are still linked or reachable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/reports is linked from the dashboard; /explore, /modules and /scorecard still build and load by URL (Scorecard badges also fail contrast: white text on green/amber).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Decide per page: remove the page and its components (ModulesView, PlacesExplorer, ReportView, PrintButton) with redirects, or keep and fix it. Update the RunDashboard links.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No dead-end or off-brand screens, and a smaller codebase for handoff.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">components/RunDashboard.tsx:69; app/(app)/{explore,modules,scorecard,reports}/page.tsx; app/(app)/scorecard/page.tsx:19-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keyboard and screen-reader users can't use the site tabs properly, and focus is invisible.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tabs are plain buttons with no tab roles, aria-selected or arrow keys; there are no focus-visible styles anywhere and .field removes the outline.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add role=tablist/tab/tabpanel, aria-selected and arrow-key handling; add focus-visible:ring-2 ring-accent to buttons, nav items and fields.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WCAG 2.2 AA keyboard and focus compliance.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">components/SiteIntelligenceTabs.tsx:204-217; app/globals.css:52-61</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Some inputs and icon buttons have no accessible label.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Intake outlet/candidate rows rely on placeholders; the location picker search and its ✕ close button have no labels.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add visible labels or aria-labels to every input and icon button.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forms work with screen readers and are clearer for older users.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">components/SteppedIntakeWizard.tsx:675-702; components/LocationPicker.tsx:131-134</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-37</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Layouts overflow on small screens.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Intake rows use a fixed grid-cols-12; the lease comps table is overflow-hidden.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use grid-cols-1 sm:grid-cols-12 for the rows; switch the table wrapper to overflow-x-auto.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The intake and the Lease tab work on phones and small laptops.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">components/SteppedIntakeWizard.tsx:674,699; components/SiteIntelligenceTabs.tsx:510</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">There are no branded loading, error or not-found screens.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No loading.tsx / error.tsx / not-found.tsx files exist, so failures show the default Next.js page.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add them under app/(app)/ in the GRID theme, with a retry action and plain-language copy.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Errors are calm, branded and recoverable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">app/(app)/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-39</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Very small text is used widely (9–11px).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">63 uses of text-[9–11px], often in muted grey — hard to read for older users.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Set a 12px minimum (13–14px for body copy); raise muted-text contrast where it sits on hover surfaces.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Readable for the older / tech-resistant audience named in the brand guidelines.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">components/SiteIntelligenceTabs.tsx; components/SteppedIntakeWizard.tsx:601</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The proxy lease corridor can't be corrected, and the map ring colour can lag the verdict.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">When no corridor matches, the Lease tab says it's a proxy but offers no picker; TerritoryMap computes its own verdict.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add a corridor picker (corridorsForRegion + corridors that have comps) that re-benchmarks; pass the blended verdict into TerritoryMap.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brokers can fix the corridor in one click, and the map always matches the verdict.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">components/SiteIntelligenceTabs.tsx; components/TerritoryMap.tsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prior backlog U-02/U-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-41</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The UI redesign has not been done yet.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Branding (palette, fonts, logo) is applied, but hierarchy, spacing and components were never designed as a system.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Run docs/DESIGN_PROMPT.md in a Claude design session, then implement the resulting tokens and component recipes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A cohesive, professional UI where the Proceed / Caution / No-Go call is obvious in under 5 seconds.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/DESIGN_PROMPT.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Owner + Dev team</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-42</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leftover AI code, config and docs remain after the AI report was removed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/ai/index.ts still lists 'vectorshift'; analysisCache/mockAnalysis/outputCheck/analysisPrompts are only used by tests; the orchestrator still deletes module='analysis' rows and site/page reads them; the PipelineUsage model remains; .env.example keeps a VectorShift section (with a real-looking pipeline id); generateGrounded writes placeholder aiGeneration rows; UI copy still says 'write-up'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Remove the unused lib/ai files and their tests; drop the vectorshift provider option; remove the 'analysis' reads/deletes; drop PipelineUsage/AiGeneration via migration (or mark them reserved); clean .env.example and UI copy; remove VECTORSHIFT_* / ANALYSIS_BACKGROUND / INTERNAL_JOB_SECRET from Netlify.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A codebase that matches the product, with no dead AI paths for the dev team to puzzle over.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/ai/*; lib/modules/orchestrator.ts:8,113; app/(app)/site/page.tsx:66; prisma/schema.prisma:592-620; .env.example</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-43</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Critical server modules have no tests.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tests cover pure math only: nothing tests orchestrator slicing/resume/failure, p2p3Modules (White-Space scope, fallbacks), territoryGuard, leaseBenchmark zonal resolution, siteFit, poiCache or the loaders; no test checks that summariseSite agrees with the scorecard; no end-to-end journey test.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add integration tests against a Neon test branch (or local Postgres + PostGIS in CI); add the verdict-agreement test; add Playwright smoke tests (login → intake → run → site tabs → PDF).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regressions are caught before deploy, and the handoff is backed by tests.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tests/unit; lib/modules/*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New audit / Prior A-04</t>
   </si>
   <si>
     <t xml:space="preserve">F-44</t>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="F7" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A7,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1999,7 +1999,7 @@
       </c>
       <c r="F9" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A9,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="F11" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A11,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="F13" s="9" t="n">
         <f aca="false">SUM(F6:F12)</f>
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2783,12 +2783,12 @@
         <v>57</v>
       </c>
       <c r="M16" s="14" t="s">
-        <v>125</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B17" s="15" t="s">
         <v>10</v>
@@ -2801,19 +2801,19 @@
         <v>P2</v>
       </c>
       <c r="E17" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="F17" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="F17" s="15" t="s">
+      <c r="G17" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="G17" s="15" t="s">
+      <c r="H17" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="H17" s="15" t="s">
+      <c r="I17" s="15" t="s">
         <v>130</v>
-      </c>
-      <c r="I17" s="15" t="s">
-        <v>131</v>
       </c>
       <c r="J17" s="14" t="s">
         <v>55</v>
@@ -2825,12 +2825,12 @@
         <v>57</v>
       </c>
       <c r="M17" s="14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>10</v>
@@ -2843,19 +2843,19 @@
         <v>P2</v>
       </c>
       <c r="E18" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="F18" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="F18" s="15" t="s">
+      <c r="G18" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="G18" s="15" t="s">
+      <c r="H18" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="H18" s="15" t="s">
+      <c r="I18" s="15" t="s">
         <v>137</v>
-      </c>
-      <c r="I18" s="15" t="s">
-        <v>138</v>
       </c>
       <c r="J18" s="14" t="s">
         <v>76</v>
@@ -2864,7 +2864,7 @@
         <v>56</v>
       </c>
       <c r="L18" s="15" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="M18" s="14" t="s">
         <v>8</v>
@@ -2872,7 +2872,7 @@
     </row>
     <row r="19" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B19" s="15" t="s">
         <v>10</v>
@@ -2885,19 +2885,19 @@
         <v>P2</v>
       </c>
       <c r="E19" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="F19" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="F19" s="15" t="s">
+      <c r="G19" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="G19" s="15" t="s">
+      <c r="H19" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="H19" s="15" t="s">
+      <c r="I19" s="15" t="s">
         <v>144</v>
-      </c>
-      <c r="I19" s="15" t="s">
-        <v>145</v>
       </c>
       <c r="J19" s="14" t="s">
         <v>76</v>
@@ -2906,7 +2906,7 @@
         <v>56</v>
       </c>
       <c r="L19" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M19" s="14" t="s">
         <v>8</v>
@@ -2914,7 +2914,7 @@
     </row>
     <row r="20" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B20" s="15" t="s">
         <v>10</v>
@@ -2927,36 +2927,36 @@
         <v>P3</v>
       </c>
       <c r="E20" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="F20" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="F20" s="15" t="s">
+      <c r="G20" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="G20" s="15" t="s">
+      <c r="H20" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="H20" s="15" t="s">
+      <c r="I20" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="I20" s="15" t="s">
+      <c r="J20" s="14" t="s">
         <v>152</v>
       </c>
-      <c r="J20" s="14" t="s">
+      <c r="K20" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="L20" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="K20" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="L20" s="15" t="s">
-        <v>154</v>
-      </c>
       <c r="M20" s="14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B21" s="15" t="s">
         <v>10</v>
@@ -2969,19 +2969,19 @@
         <v>P3</v>
       </c>
       <c r="E21" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="F21" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="F21" s="15" t="s">
+      <c r="G21" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="G21" s="15" t="s">
+      <c r="H21" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="H21" s="15" t="s">
+      <c r="I21" s="15" t="s">
         <v>159</v>
-      </c>
-      <c r="I21" s="15" t="s">
-        <v>160</v>
       </c>
       <c r="J21" s="14" t="s">
         <v>55</v>
@@ -2990,15 +2990,15 @@
         <v>46</v>
       </c>
       <c r="L21" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="M21" s="14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>10</v>
@@ -3011,19 +3011,19 @@
         <v>P3</v>
       </c>
       <c r="E22" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="F22" s="15" t="s">
         <v>163</v>
       </c>
-      <c r="F22" s="15" t="s">
+      <c r="G22" s="15" t="s">
         <v>164</v>
       </c>
-      <c r="G22" s="15" t="s">
+      <c r="H22" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="H22" s="15" t="s">
+      <c r="I22" s="15" t="s">
         <v>166</v>
-      </c>
-      <c r="I22" s="15" t="s">
-        <v>167</v>
       </c>
       <c r="J22" s="14" t="s">
         <v>76</v>
@@ -3032,7 +3032,7 @@
         <v>56</v>
       </c>
       <c r="L22" s="15" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="M22" s="14" t="s">
         <v>8</v>
@@ -3040,7 +3040,7 @@
     </row>
     <row r="23" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>10</v>
@@ -3053,36 +3053,36 @@
         <v>P1</v>
       </c>
       <c r="E23" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="F23" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="F23" s="15" t="s">
+      <c r="G23" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="G23" s="15" t="s">
+      <c r="H23" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="H23" s="15" t="s">
+      <c r="I23" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="I23" s="15" t="s">
-        <v>174</v>
-      </c>
       <c r="J23" s="14" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="K23" s="15" t="s">
         <v>46</v>
       </c>
       <c r="L23" s="15" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="M23" s="14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>11</v>
@@ -3095,19 +3095,19 @@
         <v>P1</v>
       </c>
       <c r="E24" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="F24" s="15" t="s">
         <v>177</v>
       </c>
-      <c r="F24" s="15" t="s">
+      <c r="G24" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="G24" s="15" t="s">
+      <c r="H24" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="H24" s="15" t="s">
+      <c r="I24" s="15" t="s">
         <v>180</v>
-      </c>
-      <c r="I24" s="15" t="s">
-        <v>181</v>
       </c>
       <c r="J24" s="14" t="s">
         <v>76</v>
@@ -3116,7 +3116,7 @@
         <v>56</v>
       </c>
       <c r="L24" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="M24" s="14" t="s">
         <v>8</v>
@@ -3124,7 +3124,7 @@
     </row>
     <row r="25" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B25" s="15" t="s">
         <v>11</v>
@@ -3137,19 +3137,19 @@
         <v>P2</v>
       </c>
       <c r="E25" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="F25" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="F25" s="15" t="s">
+      <c r="G25" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="G25" s="15" t="s">
+      <c r="H25" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="H25" s="15" t="s">
+      <c r="I25" s="15" t="s">
         <v>187</v>
-      </c>
-      <c r="I25" s="15" t="s">
-        <v>188</v>
       </c>
       <c r="J25" s="14" t="s">
         <v>55</v>
@@ -3166,7 +3166,7 @@
     </row>
     <row r="26" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>11</v>
@@ -3179,19 +3179,19 @@
         <v>P2</v>
       </c>
       <c r="E26" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="F26" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="F26" s="15" t="s">
+      <c r="G26" s="15" t="s">
         <v>191</v>
       </c>
-      <c r="G26" s="15" t="s">
+      <c r="H26" s="15" t="s">
         <v>192</v>
       </c>
-      <c r="H26" s="15" t="s">
+      <c r="I26" s="15" t="s">
         <v>193</v>
-      </c>
-      <c r="I26" s="15" t="s">
-        <v>194</v>
       </c>
       <c r="J26" s="14" t="s">
         <v>76</v>
@@ -3200,7 +3200,7 @@
         <v>56</v>
       </c>
       <c r="L26" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M26" s="14" t="s">
         <v>8</v>
@@ -3208,7 +3208,7 @@
     </row>
     <row r="27" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B27" s="15" t="s">
         <v>11</v>
@@ -3221,19 +3221,19 @@
         <v>P3</v>
       </c>
       <c r="E27" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="F27" s="15" t="s">
         <v>197</v>
       </c>
-      <c r="F27" s="15" t="s">
+      <c r="G27" s="15" t="s">
         <v>198</v>
       </c>
-      <c r="G27" s="15" t="s">
+      <c r="H27" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="H27" s="15" t="s">
+      <c r="I27" s="15" t="s">
         <v>200</v>
-      </c>
-      <c r="I27" s="15" t="s">
-        <v>201</v>
       </c>
       <c r="J27" s="14" t="s">
         <v>55</v>
@@ -3250,7 +3250,7 @@
     </row>
     <row r="28" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>12</v>
@@ -3263,19 +3263,19 @@
         <v>P2</v>
       </c>
       <c r="E28" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="F28" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="F28" s="15" t="s">
+      <c r="G28" s="15" t="s">
         <v>204</v>
       </c>
-      <c r="G28" s="15" t="s">
+      <c r="H28" s="15" t="s">
         <v>205</v>
       </c>
-      <c r="H28" s="15" t="s">
+      <c r="I28" s="15" t="s">
         <v>206</v>
-      </c>
-      <c r="I28" s="15" t="s">
-        <v>207</v>
       </c>
       <c r="J28" s="14" t="s">
         <v>55</v>
@@ -3292,7 +3292,7 @@
     </row>
     <row r="29" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B29" s="15" t="s">
         <v>12</v>
@@ -3305,19 +3305,19 @@
         <v>P2</v>
       </c>
       <c r="E29" s="15" t="s">
+        <v>208</v>
+      </c>
+      <c r="F29" s="15" t="s">
         <v>209</v>
       </c>
-      <c r="F29" s="15" t="s">
+      <c r="G29" s="15" t="s">
         <v>210</v>
       </c>
-      <c r="G29" s="15" t="s">
+      <c r="H29" s="15" t="s">
         <v>211</v>
       </c>
-      <c r="H29" s="15" t="s">
+      <c r="I29" s="15" t="s">
         <v>212</v>
-      </c>
-      <c r="I29" s="15" t="s">
-        <v>213</v>
       </c>
       <c r="J29" s="14" t="s">
         <v>76</v>
@@ -3329,12 +3329,12 @@
         <v>57</v>
       </c>
       <c r="M29" s="14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="14" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B30" s="15" t="s">
         <v>12</v>
@@ -3347,19 +3347,19 @@
         <v>P2</v>
       </c>
       <c r="E30" s="15" t="s">
+        <v>214</v>
+      </c>
+      <c r="F30" s="15" t="s">
         <v>215</v>
       </c>
-      <c r="F30" s="15" t="s">
+      <c r="G30" s="15" t="s">
         <v>216</v>
       </c>
-      <c r="G30" s="15" t="s">
+      <c r="H30" s="15" t="s">
         <v>217</v>
       </c>
-      <c r="H30" s="15" t="s">
+      <c r="I30" s="15" t="s">
         <v>218</v>
-      </c>
-      <c r="I30" s="15" t="s">
-        <v>219</v>
       </c>
       <c r="J30" s="14" t="s">
         <v>76</v>
@@ -3368,15 +3368,15 @@
         <v>56</v>
       </c>
       <c r="L30" s="15" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="M30" s="14" t="s">
-        <v>132</v>
+        <v>8</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B31" s="15" t="s">
         <v>12</v>
@@ -3389,19 +3389,19 @@
         <v>P2</v>
       </c>
       <c r="E31" s="15" t="s">
+        <v>221</v>
+      </c>
+      <c r="F31" s="15" t="s">
         <v>222</v>
       </c>
-      <c r="F31" s="15" t="s">
+      <c r="G31" s="15" t="s">
         <v>223</v>
       </c>
-      <c r="G31" s="15" t="s">
+      <c r="H31" s="15" t="s">
         <v>224</v>
       </c>
-      <c r="H31" s="15" t="s">
+      <c r="I31" s="15" t="s">
         <v>225</v>
-      </c>
-      <c r="I31" s="15" t="s">
-        <v>226</v>
       </c>
       <c r="J31" s="14" t="s">
         <v>55</v>
@@ -3418,7 +3418,7 @@
     </row>
     <row r="32" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="14" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>12</v>
@@ -3431,19 +3431,19 @@
         <v>P2</v>
       </c>
       <c r="E32" s="15" t="s">
+        <v>227</v>
+      </c>
+      <c r="F32" s="15" t="s">
         <v>228</v>
       </c>
-      <c r="F32" s="15" t="s">
+      <c r="G32" s="15" t="s">
         <v>229</v>
       </c>
-      <c r="G32" s="15" t="s">
+      <c r="H32" s="15" t="s">
         <v>230</v>
       </c>
-      <c r="H32" s="15" t="s">
+      <c r="I32" s="15" t="s">
         <v>231</v>
-      </c>
-      <c r="I32" s="15" t="s">
-        <v>232</v>
       </c>
       <c r="J32" s="14" t="s">
         <v>55</v>
@@ -3460,7 +3460,7 @@
     </row>
     <row r="33" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B33" s="15" t="s">
         <v>12</v>
@@ -3473,19 +3473,19 @@
         <v>P3</v>
       </c>
       <c r="E33" s="15" t="s">
+        <v>233</v>
+      </c>
+      <c r="F33" s="15" t="s">
         <v>234</v>
       </c>
-      <c r="F33" s="15" t="s">
+      <c r="G33" s="15" t="s">
         <v>235</v>
       </c>
-      <c r="G33" s="15" t="s">
+      <c r="H33" s="15" t="s">
         <v>236</v>
       </c>
-      <c r="H33" s="15" t="s">
+      <c r="I33" s="15" t="s">
         <v>237</v>
-      </c>
-      <c r="I33" s="15" t="s">
-        <v>238</v>
       </c>
       <c r="J33" s="14" t="s">
         <v>55</v>
@@ -3502,7 +3502,7 @@
     </row>
     <row r="34" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B34" s="15" t="s">
         <v>12</v>
@@ -3515,19 +3515,19 @@
         <v>P2</v>
       </c>
       <c r="E34" s="15" t="s">
+        <v>239</v>
+      </c>
+      <c r="F34" s="15" t="s">
         <v>240</v>
       </c>
-      <c r="F34" s="15" t="s">
+      <c r="G34" s="15" t="s">
         <v>241</v>
       </c>
-      <c r="G34" s="15" t="s">
+      <c r="H34" s="15" t="s">
         <v>242</v>
       </c>
-      <c r="H34" s="15" t="s">
+      <c r="I34" s="15" t="s">
         <v>243</v>
-      </c>
-      <c r="I34" s="15" t="s">
-        <v>244</v>
       </c>
       <c r="J34" s="14" t="s">
         <v>76</v>
@@ -3536,15 +3536,15 @@
         <v>56</v>
       </c>
       <c r="L34" s="15" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="M34" s="14" t="s">
-        <v>132</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B35" s="15" t="s">
         <v>12</v>
@@ -3557,19 +3557,19 @@
         <v>P1</v>
       </c>
       <c r="E35" s="15" t="s">
+        <v>246</v>
+      </c>
+      <c r="F35" s="15" t="s">
         <v>247</v>
       </c>
-      <c r="F35" s="15" t="s">
+      <c r="G35" s="15" t="s">
         <v>248</v>
       </c>
-      <c r="G35" s="15" t="s">
+      <c r="H35" s="15" t="s">
         <v>249</v>
       </c>
-      <c r="H35" s="15" t="s">
+      <c r="I35" s="15" t="s">
         <v>250</v>
-      </c>
-      <c r="I35" s="15" t="s">
-        <v>251</v>
       </c>
       <c r="J35" s="14" t="s">
         <v>55</v>
@@ -3578,15 +3578,15 @@
         <v>46</v>
       </c>
       <c r="L35" s="15" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="M35" s="14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B36" s="15" t="s">
         <v>13</v>
@@ -3599,19 +3599,19 @@
         <v>P1</v>
       </c>
       <c r="E36" s="15" t="s">
+        <v>253</v>
+      </c>
+      <c r="F36" s="15" t="s">
         <v>254</v>
       </c>
-      <c r="F36" s="15" t="s">
+      <c r="G36" s="15" t="s">
         <v>255</v>
       </c>
-      <c r="G36" s="15" t="s">
+      <c r="H36" s="15" t="s">
         <v>256</v>
       </c>
-      <c r="H36" s="15" t="s">
+      <c r="I36" s="15" t="s">
         <v>257</v>
-      </c>
-      <c r="I36" s="15" t="s">
-        <v>258</v>
       </c>
       <c r="J36" s="14" t="s">
         <v>55</v>
@@ -3620,7 +3620,7 @@
         <v>56</v>
       </c>
       <c r="L36" s="15" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="M36" s="14" t="s">
         <v>8</v>
@@ -3628,7 +3628,7 @@
     </row>
     <row r="37" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B37" s="15" t="s">
         <v>13</v>
@@ -3641,19 +3641,19 @@
         <v>P1</v>
       </c>
       <c r="E37" s="15" t="s">
+        <v>260</v>
+      </c>
+      <c r="F37" s="15" t="s">
         <v>261</v>
       </c>
-      <c r="F37" s="15" t="s">
+      <c r="G37" s="15" t="s">
         <v>262</v>
       </c>
-      <c r="G37" s="15" t="s">
+      <c r="H37" s="15" t="s">
         <v>263</v>
       </c>
-      <c r="H37" s="15" t="s">
+      <c r="I37" s="15" t="s">
         <v>264</v>
-      </c>
-      <c r="I37" s="15" t="s">
-        <v>265</v>
       </c>
       <c r="J37" s="14" t="s">
         <v>55</v>
@@ -3670,7 +3670,7 @@
     </row>
     <row r="38" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="14" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B38" s="15" t="s">
         <v>13</v>
@@ -3683,19 +3683,19 @@
         <v>P2</v>
       </c>
       <c r="E38" s="15" t="s">
+        <v>266</v>
+      </c>
+      <c r="F38" s="15" t="s">
         <v>267</v>
       </c>
-      <c r="F38" s="15" t="s">
+      <c r="G38" s="15" t="s">
         <v>268</v>
       </c>
-      <c r="G38" s="15" t="s">
+      <c r="H38" s="15" t="s">
         <v>269</v>
       </c>
-      <c r="H38" s="15" t="s">
+      <c r="I38" s="15" t="s">
         <v>270</v>
-      </c>
-      <c r="I38" s="15" t="s">
-        <v>271</v>
       </c>
       <c r="J38" s="14" t="s">
         <v>55</v>
@@ -3712,7 +3712,7 @@
     </row>
     <row r="39" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="14" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B39" s="15" t="s">
         <v>13</v>
@@ -3725,19 +3725,19 @@
         <v>P2</v>
       </c>
       <c r="E39" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="F39" s="15" t="s">
         <v>273</v>
       </c>
-      <c r="F39" s="15" t="s">
+      <c r="G39" s="15" t="s">
         <v>274</v>
       </c>
-      <c r="G39" s="15" t="s">
+      <c r="H39" s="15" t="s">
         <v>275</v>
       </c>
-      <c r="H39" s="15" t="s">
+      <c r="I39" s="15" t="s">
         <v>276</v>
-      </c>
-      <c r="I39" s="15" t="s">
-        <v>277</v>
       </c>
       <c r="J39" s="14" t="s">
         <v>55</v>
@@ -3754,7 +3754,7 @@
     </row>
     <row r="40" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B40" s="15" t="s">
         <v>13</v>
@@ -3767,19 +3767,19 @@
         <v>P2</v>
       </c>
       <c r="E40" s="15" t="s">
+        <v>278</v>
+      </c>
+      <c r="F40" s="15" t="s">
         <v>279</v>
       </c>
-      <c r="F40" s="15" t="s">
+      <c r="G40" s="15" t="s">
         <v>280</v>
       </c>
-      <c r="G40" s="15" t="s">
+      <c r="H40" s="15" t="s">
         <v>281</v>
       </c>
-      <c r="H40" s="15" t="s">
+      <c r="I40" s="15" t="s">
         <v>282</v>
-      </c>
-      <c r="I40" s="15" t="s">
-        <v>283</v>
       </c>
       <c r="J40" s="14" t="s">
         <v>55</v>
@@ -3796,7 +3796,7 @@
     </row>
     <row r="41" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B41" s="15" t="s">
         <v>13</v>
@@ -3809,19 +3809,19 @@
         <v>P2</v>
       </c>
       <c r="E41" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="F41" s="15" t="s">
         <v>285</v>
       </c>
-      <c r="F41" s="15" t="s">
+      <c r="G41" s="15" t="s">
         <v>286</v>
       </c>
-      <c r="G41" s="15" t="s">
+      <c r="H41" s="15" t="s">
         <v>287</v>
       </c>
-      <c r="H41" s="15" t="s">
+      <c r="I41" s="15" t="s">
         <v>288</v>
-      </c>
-      <c r="I41" s="15" t="s">
-        <v>289</v>
       </c>
       <c r="J41" s="14" t="s">
         <v>55</v>
@@ -3838,7 +3838,7 @@
     </row>
     <row r="42" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="14" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B42" s="15" t="s">
         <v>13</v>
@@ -3851,19 +3851,19 @@
         <v>P2</v>
       </c>
       <c r="E42" s="15" t="s">
+        <v>290</v>
+      </c>
+      <c r="F42" s="15" t="s">
         <v>291</v>
       </c>
-      <c r="F42" s="15" t="s">
+      <c r="G42" s="15" t="s">
         <v>292</v>
       </c>
-      <c r="G42" s="15" t="s">
+      <c r="H42" s="15" t="s">
         <v>293</v>
       </c>
-      <c r="H42" s="15" t="s">
+      <c r="I42" s="15" t="s">
         <v>294</v>
-      </c>
-      <c r="I42" s="15" t="s">
-        <v>295</v>
       </c>
       <c r="J42" s="14" t="s">
         <v>55</v>
@@ -3880,7 +3880,7 @@
     </row>
     <row r="43" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="14" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B43" s="15" t="s">
         <v>13</v>
@@ -3893,19 +3893,19 @@
         <v>P2</v>
       </c>
       <c r="E43" s="15" t="s">
+        <v>296</v>
+      </c>
+      <c r="F43" s="15" t="s">
         <v>297</v>
       </c>
-      <c r="F43" s="15" t="s">
+      <c r="G43" s="15" t="s">
         <v>298</v>
       </c>
-      <c r="G43" s="15" t="s">
+      <c r="H43" s="15" t="s">
         <v>299</v>
       </c>
-      <c r="H43" s="15" t="s">
+      <c r="I43" s="15" t="s">
         <v>300</v>
-      </c>
-      <c r="I43" s="15" t="s">
-        <v>301</v>
       </c>
       <c r="J43" s="14" t="s">
         <v>76</v>
@@ -3922,7 +3922,7 @@
     </row>
     <row r="44" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="14" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B44" s="15" t="s">
         <v>13</v>
@@ -3935,19 +3935,19 @@
         <v>P2</v>
       </c>
       <c r="E44" s="15" t="s">
+        <v>302</v>
+      </c>
+      <c r="F44" s="15" t="s">
         <v>303</v>
       </c>
-      <c r="F44" s="15" t="s">
+      <c r="G44" s="15" t="s">
         <v>304</v>
       </c>
-      <c r="G44" s="15" t="s">
+      <c r="H44" s="15" t="s">
         <v>305</v>
       </c>
-      <c r="H44" s="15" t="s">
+      <c r="I44" s="15" t="s">
         <v>306</v>
-      </c>
-      <c r="I44" s="15" t="s">
-        <v>307</v>
       </c>
       <c r="J44" s="14" t="s">
         <v>55</v>
@@ -3956,7 +3956,7 @@
         <v>56</v>
       </c>
       <c r="L44" s="15" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="M44" s="14" t="s">
         <v>8</v>
@@ -3964,7 +3964,7 @@
     </row>
     <row r="45" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="14" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B45" s="15" t="s">
         <v>13</v>
@@ -3977,25 +3977,25 @@
         <v>P2</v>
       </c>
       <c r="E45" s="15" t="s">
+        <v>309</v>
+      </c>
+      <c r="F45" s="15" t="s">
         <v>310</v>
       </c>
-      <c r="F45" s="15" t="s">
+      <c r="G45" s="15" t="s">
         <v>311</v>
       </c>
-      <c r="G45" s="15" t="s">
+      <c r="H45" s="15" t="s">
         <v>312</v>
       </c>
-      <c r="H45" s="15" t="s">
+      <c r="I45" s="15" t="s">
         <v>313</v>
       </c>
-      <c r="I45" s="15" t="s">
+      <c r="J45" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="K45" s="15" t="s">
         <v>314</v>
-      </c>
-      <c r="J45" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="K45" s="15" t="s">
-        <v>315</v>
       </c>
       <c r="L45" s="15" t="s">
         <v>57</v>
@@ -4006,7 +4006,7 @@
     </row>
     <row r="46" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="14" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B46" s="15" t="s">
         <v>14</v>
@@ -4019,19 +4019,19 @@
         <v>P2</v>
       </c>
       <c r="E46" s="15" t="s">
+        <v>316</v>
+      </c>
+      <c r="F46" s="15" t="s">
         <v>317</v>
       </c>
-      <c r="F46" s="15" t="s">
+      <c r="G46" s="15" t="s">
         <v>318</v>
       </c>
-      <c r="G46" s="15" t="s">
+      <c r="H46" s="15" t="s">
         <v>319</v>
       </c>
-      <c r="H46" s="15" t="s">
+      <c r="I46" s="15" t="s">
         <v>320</v>
-      </c>
-      <c r="I46" s="15" t="s">
-        <v>321</v>
       </c>
       <c r="J46" s="14" t="s">
         <v>76</v>
@@ -4043,12 +4043,12 @@
         <v>57</v>
       </c>
       <c r="M46" s="14" t="s">
-        <v>125</v>
+        <v>8</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="14" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B47" s="15" t="s">
         <v>14</v>
@@ -4061,31 +4061,31 @@
         <v>P2</v>
       </c>
       <c r="E47" s="15" t="s">
+        <v>322</v>
+      </c>
+      <c r="F47" s="15" t="s">
         <v>323</v>
       </c>
-      <c r="F47" s="15" t="s">
+      <c r="G47" s="15" t="s">
         <v>324</v>
       </c>
-      <c r="G47" s="15" t="s">
+      <c r="H47" s="15" t="s">
         <v>325</v>
       </c>
-      <c r="H47" s="15" t="s">
+      <c r="I47" s="15" t="s">
         <v>326</v>
       </c>
-      <c r="I47" s="15" t="s">
+      <c r="J47" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="K47" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="L47" s="15" t="s">
         <v>327</v>
       </c>
-      <c r="J47" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="K47" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="L47" s="15" t="s">
+      <c r="M47" s="14" t="s">
         <v>328</v>
-      </c>
-      <c r="M47" s="14" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4127,7 +4127,7 @@
         <v>57</v>
       </c>
       <c r="M48" s="14" t="s">
-        <v>132</v>
+        <v>328</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4211,7 +4211,7 @@
         <v>347</v>
       </c>
       <c r="M50" s="14" t="s">
-        <v>132</v>
+        <v>328</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4253,7 +4253,7 @@
         <v>354</v>
       </c>
       <c r="M51" s="14" t="s">
-        <v>132</v>
+        <v>8</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4421,7 +4421,7 @@
         <v>382</v>
       </c>
       <c r="M55" s="14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4463,7 +4463,7 @@
         <v>57</v>
       </c>
       <c r="M56" s="14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
complete audit: lease loader safety (F-13), Google API quotas+bounds (F-25), monitoring seam + client-error (F-51), Playwright CI smoke + service tests (F-43), lint cleanups (F-46), docs refresh + owner runbook (F-52, F-16/17/19/31)
</commit_message>
<xml_diff>
--- a/docs/BSA_Application_Audit.xlsx
+++ b/docs/BSA_Application_Audit.xlsx
@@ -420,75 +420,75 @@
     <t xml:space="preserve">lib/ingest/loaders.ts:112-133</t>
   </si>
   <si>
+    <t xml:space="preserve">F-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lease comps have no freshness rule.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">observedDate is only used for ordering; old comps are never flagged or aged out.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flag comps older than 18 months, down-weight or exclude them past 36 months, and show 'data as of' on the Lease tab. Optional broker endpoint to submit confirmed rents.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rent benchmarks reflect the current market and say how recent they are.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/modules/leaseBenchmark.ts:122-153</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior backlog D-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Site Fit 'accessibility' pillar is always empty.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No transport layer is loaded, so the 15% accessibility pillar is null for every site.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load OSM transport features (jeepney/bus stops, rail stations, major roads) per region and score distance/density to them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site Fit reflects how easy a site is to reach — important for Filipino commuter traffic.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/modules/siteFit.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior backlog D-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trade areas are fixed circles.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catchments are circles by format (600–1,200 m); rivers, highways and gated areas are ignored.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use travel-time isochrones (self-hosted OSRM/Valhalla or an isochrone API), cached per site.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catchments match how customers actually reach the site.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lib/modules/territoryMath.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior backlog D-02</t>
+  </si>
+  <si>
     <t xml:space="preserve">Open</t>
   </si>
   <si>
-    <t xml:space="preserve">F-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lease comps have no freshness rule.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">observedDate is only used for ordering; old comps are never flagged or aged out.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flag comps older than 18 months, down-weight or exclude them past 36 months, and show 'data as of' on the Lease tab. Optional broker endpoint to submit confirmed rents.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rent benchmarks reflect the current market and say how recent they are.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/modules/leaseBenchmark.ts:122-153</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prior backlog D-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Site Fit 'accessibility' pillar is always empty.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No transport layer is loaded, so the 15% accessibility pillar is null for every site.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Load OSM transport features (jeepney/bus stops, rail stations, major roads) per region and score distance/density to them.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Site Fit reflects how easy a site is to reach — important for Filipino commuter traffic.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/modules/siteFit.ts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prior backlog D-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trade areas are fixed circles.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Catchments are circles by format (600–1,200 m); rivers, highways and gated areas are ignored.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use travel-time isochrones (self-hosted OSRM/Valhalla or an isochrone API), cached per site.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Catchments match how customers actually reach the site.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lib/modules/territoryMath.ts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prior backlog D-02</t>
-  </si>
-  <si>
     <t xml:space="preserve">F-17</t>
   </si>
   <si>
@@ -1011,25 +1011,25 @@
     <t xml:space="preserve">New audit / Prior A-04</t>
   </si>
   <si>
+    <t xml:space="preserve">F-44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very large components are hard to maintain.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SiteIntelligenceTabs.tsx (~1,100 lines), SteppedIntakeWizard.tsx (~750), FranchiseScreeningView.tsx (~600).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Split each tab and wizard step into its own file; move shared tone maps and chips to components/ui.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Smaller, reviewable files that the dev team can work on in parallel.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">components/SiteIntelligenceTabs.tsx; components/SteppedIntakeWizard.tsx; components/FranchiseScreeningView.tsx</t>
+  </si>
+  <si>
     <t xml:space="preserve">In progress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-44</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Very large components are hard to maintain.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SiteIntelligenceTabs.tsx (~1,100 lines), SteppedIntakeWizard.tsx (~750), FranchiseScreeningView.tsx (~600).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Split each tab and wizard step into its own file; move shared tone maps and chips to components/ui.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Smaller, reviewable files that the dev team can work on in parallel.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">components/SiteIntelligenceTabs.tsx; components/SteppedIntakeWizard.tsx; components/FranchiseScreeningView.tsx</t>
   </si>
   <si>
     <t xml:space="preserve">F-45</t>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="F7" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A7,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1999,7 +1999,7 @@
       </c>
       <c r="F9" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A9,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="F11" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A11,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="F12" s="7" t="n">
         <f aca="false">COUNTIFS('Audit Findings'!$B$5:$B$56,$A12,'Audit Findings'!$M$5:$M$56,"Done")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="F13" s="9" t="n">
         <f aca="false">SUM(F6:F12)</f>
-        <v>41</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2825,12 +2825,12 @@
         <v>57</v>
       </c>
       <c r="M17" s="14" t="s">
-        <v>131</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B18" s="15" t="s">
         <v>10</v>
@@ -2843,19 +2843,19 @@
         <v>P2</v>
       </c>
       <c r="E18" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="F18" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="F18" s="15" t="s">
+      <c r="G18" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="G18" s="15" t="s">
+      <c r="H18" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="H18" s="15" t="s">
+      <c r="I18" s="15" t="s">
         <v>136</v>
-      </c>
-      <c r="I18" s="15" t="s">
-        <v>137</v>
       </c>
       <c r="J18" s="14" t="s">
         <v>76</v>
@@ -2864,7 +2864,7 @@
         <v>56</v>
       </c>
       <c r="L18" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="M18" s="14" t="s">
         <v>8</v>
@@ -2872,7 +2872,7 @@
     </row>
     <row r="19" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B19" s="15" t="s">
         <v>10</v>
@@ -2885,19 +2885,19 @@
         <v>P2</v>
       </c>
       <c r="E19" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="F19" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="F19" s="15" t="s">
+      <c r="G19" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="G19" s="15" t="s">
+      <c r="H19" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="H19" s="15" t="s">
+      <c r="I19" s="15" t="s">
         <v>143</v>
-      </c>
-      <c r="I19" s="15" t="s">
-        <v>144</v>
       </c>
       <c r="J19" s="14" t="s">
         <v>76</v>
@@ -2906,7 +2906,7 @@
         <v>56</v>
       </c>
       <c r="L19" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="M19" s="14" t="s">
         <v>8</v>
@@ -2914,7 +2914,7 @@
     </row>
     <row r="20" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B20" s="15" t="s">
         <v>10</v>
@@ -2927,31 +2927,31 @@
         <v>P3</v>
       </c>
       <c r="E20" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="F20" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="F20" s="15" t="s">
+      <c r="G20" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="G20" s="15" t="s">
+      <c r="H20" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="H20" s="15" t="s">
+      <c r="I20" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="I20" s="15" t="s">
+      <c r="J20" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="J20" s="14" t="s">
+      <c r="K20" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="L20" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="K20" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="L20" s="15" t="s">
+      <c r="M20" s="14" t="s">
         <v>153</v>
-      </c>
-      <c r="M20" s="14" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2993,7 +2993,7 @@
         <v>160</v>
       </c>
       <c r="M21" s="14" t="s">
-        <v>131</v>
+        <v>153</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3068,7 +3068,7 @@
         <v>173</v>
       </c>
       <c r="J23" s="14" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K23" s="15" t="s">
         <v>46</v>
@@ -3077,7 +3077,7 @@
         <v>174</v>
       </c>
       <c r="M23" s="14" t="s">
-        <v>131</v>
+        <v>153</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3329,7 +3329,7 @@
         <v>57</v>
       </c>
       <c r="M29" s="14" t="s">
-        <v>131</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3581,7 +3581,7 @@
         <v>251</v>
       </c>
       <c r="M35" s="14" t="s">
-        <v>131</v>
+        <v>153</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3992,7 +3992,7 @@
         <v>313</v>
       </c>
       <c r="J45" s="14" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K45" s="15" t="s">
         <v>314</v>
@@ -4076,7 +4076,7 @@
         <v>326</v>
       </c>
       <c r="J47" s="14" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K47" s="15" t="s">
         <v>56</v>
@@ -4085,12 +4085,12 @@
         <v>327</v>
       </c>
       <c r="M47" s="14" t="s">
-        <v>328</v>
+        <v>8</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="14" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B48" s="15" t="s">
         <v>14</v>
@@ -4103,19 +4103,19 @@
         <v>P3</v>
       </c>
       <c r="E48" s="15" t="s">
+        <v>329</v>
+      </c>
+      <c r="F48" s="15" t="s">
         <v>330</v>
       </c>
-      <c r="F48" s="15" t="s">
+      <c r="G48" s="15" t="s">
         <v>331</v>
       </c>
-      <c r="G48" s="15" t="s">
+      <c r="H48" s="15" t="s">
         <v>332</v>
       </c>
-      <c r="H48" s="15" t="s">
+      <c r="I48" s="15" t="s">
         <v>333</v>
-      </c>
-      <c r="I48" s="15" t="s">
-        <v>334</v>
       </c>
       <c r="J48" s="14" t="s">
         <v>76</v>
@@ -4127,7 +4127,7 @@
         <v>57</v>
       </c>
       <c r="M48" s="14" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4211,7 +4211,7 @@
         <v>347</v>
       </c>
       <c r="M50" s="14" t="s">
-        <v>328</v>
+        <v>8</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4421,7 +4421,7 @@
         <v>382</v>
       </c>
       <c r="M55" s="14" t="s">
-        <v>131</v>
+        <v>8</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4463,7 +4463,7 @@
         <v>57</v>
       </c>
       <c r="M56" s="14" t="s">
-        <v>131</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>